<commit_message>
se modifico todo el sistema
</commit_message>
<xml_diff>
--- a/scripts/evaluacion/data/data.xlsx
+++ b/scripts/evaluacion/data/data.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:L51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,35 +451,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>fuente_kcal</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>texto_ref</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>texto_rag</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>score_similitud</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>chunks_recuperados</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>tokens_entrada</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>tokens_salida</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>tiempo_ms</t>
         </is>
@@ -500,38 +505,37 @@
         <v>351</v>
       </c>
       <c r="D2" t="n">
-        <v>337</v>
+        <v>89</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>La quinua contiene 351 kcal por 100g según la TPCA CENAN/INS 2025. Aporta 13.6g de proteínas, 5.8g de grasas y 66.6g de carbohidratos disponibles. Tiene 5.9g de fibra dietaria. Es un alimento de alto valor nutricional.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, la quinua tiene diferentes valores de calorías por 100 gramos dependiendo de su forma y variedad:
-- Quinua, harina de: 337.0 kcal
-- Quinua cocida: 89.0 kcal
-- Quinua: 351.0 kcal
-- Quinua, variedad real: 331.0 kcal
-- Quinua, variedad CICA-127 (Puno): 360.0 kcal
-Estos valores pueden variar ligeramente dependiendo de la variedad de quinua y su forma de preparación.</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>0.8813</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>La quinua contiene 351 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H2" t="n">
-        <v>5</v>
+        <v>0.6945</v>
       </c>
       <c r="I2" t="n">
-        <v>3579</v>
+        <v>7</v>
       </c>
       <c r="J2" t="n">
-        <v>150</v>
+        <v>3841</v>
       </c>
       <c r="K2" t="n">
-        <v>9582</v>
+        <v>21</v>
+      </c>
+      <c r="L2" t="n">
+        <v>6302.8</v>
       </c>
     </row>
     <row r="3">
@@ -549,41 +553,41 @@
         <v>351</v>
       </c>
       <c r="D3" t="n">
-        <v>351</v>
+        <v>361</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
           <t>La quinua por 100g aporta 351 kcal, 13.6g de proteínas de alto valor biológico, 5.8g de grasas totales y 66.6g de carbohidratos según la TPCA CENAN/INS. Contiene los 9 aminoácidos esenciales. Su fibra dietaria de 5.9g favorece el control glucémico.</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>La quinua es un alimento muy nutritivo y recomendado para personas con diabetes tipo 2 debido a su bajo Índice Glucémico (IG=53) y su alto contenido de fibra. Aquí te presento el perfil de macronutrientes de la quinua según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS:
-🌾 **Quinua**
-- Energía: 351.0 kcal
-- Proteínas: 13.6g
-- Grasas: 5.8g
-- Carbohidratos totales: 66.6g
-- Carbohidratos disponibles: 60.7g
-- Fibra dietaria: 5.9g
-La quinua es una excelente fuente de proteínas vegetales y fibra dietaria. La fibra ayuda a ralentizar la absorción de azúcar en el torrente sanguíneo, lo que puede ayudar a controlar los niveles de glucosa en la sangre. Además, la quinua es una buena opción para las personas que siguen una dieta vegetariana o vegana, ya que proporciona una fuente completa de proteínas. 
-Recuerda siempre controlar las porciones, ya que aunque la quinua es saludable, también es densa en energía. Una porción adecuada para una comida es de aproximadamente 1/3 a 1/2 taza de quinua cocida.</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>0.844</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>La quinua contiene 351 kcal por 100g según la TPCA CENAN/INS. Aquí tienes el perfil completo de macronutrientes:
+- **Proteínas:** 13.6g
+- **Grasas:** 5.8g
+- **Carbohidratos:** 66.6g
+Además, la quinua es una excelente fuente de fibra, con 5.9g por cada 100g. ¡Es un alimento muy nutritivo y recomendado para personas con diabetes tipo 2!</t>
+        </is>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>0.6267</v>
       </c>
       <c r="I3" t="n">
-        <v>3556</v>
+        <v>9</v>
       </c>
       <c r="J3" t="n">
-        <v>331</v>
+        <v>4497</v>
       </c>
       <c r="K3" t="n">
-        <v>8598</v>
+        <v>108</v>
+      </c>
+      <c r="L3" t="n">
+        <v>7026.2</v>
       </c>
     </row>
     <row r="4">
@@ -601,38 +605,38 @@
         <v>351</v>
       </c>
       <c r="D4" t="n">
-        <v>89</v>
+        <v>337</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
           <t>La quinua contiene 351 kcal por 100g según la TPCA. Su índice glucémico es 53, moderado-bajo. Es RECOMENDADA para DM2 porque su alta proteína (13.6g) y fibra (5.9g) reducen el pico glucémico postprandial. Sustituye al arroz blanco (IG 73) como fuente de carbohidratos.</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>La quinua es un alimento muy nutritivo y recomendado para pacientes con diabetes tipo 2 por varias razones. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, la quinua cocida tiene 89.0 kcal por cada 100g de porción comestible. 
-Aquí te explico por qué es recomendada:
-1. **Índice Glucémico (IG) bajo:** La quinua tiene un IG de 53, lo que significa que sus carbohidratos se absorben lentamente, evitando picos bruscos de glucosa en la sangre, lo cual es beneficioso para controlar la diabetes.
-2. **Rica en fibra:** La fibra ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo, lo que contribuye a mantener niveles estables de azúcar en la sangre.
-3. **Proteínas:** La quinua es una excelente fuente de proteínas, lo que puede ayudar a controlar el hambre y mantener la masa muscular.
-4. **Nutrientes esenciales:** Además, la quinua es rica en vitaminas y minerales como el hierro y el calcio, y es una excelente fuente de fósforo, un mineral que ayuda a reparar células y tejidos en el cuerpo.
-Recuerda que aunque la quinua es un alimento saludable, su consumo debe ser moderado y dentro de una dieta equilibrada, ya que también aporta carbohidratos. Para un control adecuado de la diabetes, es importante considerar la cantidad total de carbohidratos en la dieta, no solo el tipo de carbohidrato.</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>0.8521</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>La quinua contiene 351 kcal por 100g según la TPCA CENAN/INS. 
+Es recomendada para pacientes con diabetes tipo 2 porque tiene un Índice Glucémico (IG) de 53, lo que significa que su impacto en los niveles de glucosa en sangre es bajo. Además, la quinua es rica en proteínas (13.6g por 100g) y fibra (5.9g por 100g), lo que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo, evitando picos de azúcar. Esto es crucial para el manejo de la diabetes tipo 2, ya que promueve un control más estable de la glucemia. Según la TPCA del CENAN/INS, la quinua es un alimento nutritivo y seguro para incluir en la dieta de personas con diabetes.</t>
+        </is>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>0.6304999999999999</v>
       </c>
       <c r="I4" t="n">
-        <v>3431</v>
+        <v>10</v>
       </c>
       <c r="J4" t="n">
-        <v>392</v>
+        <v>4669</v>
       </c>
       <c r="K4" t="n">
-        <v>15596</v>
+        <v>179</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9548.700000000001</v>
       </c>
     </row>
     <row r="5">
@@ -650,32 +654,37 @@
         <v>399</v>
       </c>
       <c r="D5" t="n">
-        <v>343</v>
+        <v>242</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
           <t>El tarwi o chocho crudo contiene 399 kcal por 100g según la TPCA CENAN/INS 2025. Es el alimento andino con mayor contenido proteico: 47.0g de proteínas por 100g. Aporta 21.3g de grasas y solo 16.5g de carbohidratos.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>El tarwi o chocho crudo tiene 343.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú. Este alimento es una excelente fuente de proteína vegetal y fibra, y tiene un Índice Glucémico (IG) muy bajo de 15, lo que lo hace muy recomendable para personas con Diabetes Mellitus Tipo 2.</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>0.8344</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>El tarwi (chocho) contiene 364 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H5" t="n">
-        <v>5</v>
+        <v>0.5487</v>
       </c>
       <c r="I5" t="n">
-        <v>3434</v>
+        <v>6</v>
       </c>
       <c r="J5" t="n">
-        <v>114</v>
+        <v>3347</v>
       </c>
       <c r="K5" t="n">
-        <v>7097</v>
+        <v>25</v>
+      </c>
+      <c r="L5" t="n">
+        <v>7048.9</v>
       </c>
     </row>
     <row r="6">
@@ -693,38 +702,38 @@
         <v>399</v>
       </c>
       <c r="D6" t="n">
-        <v>343</v>
+        <v>115</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>El tarwi contiene 399 kcal y 47.0g de proteínas por 100g, siendo la leguminosa andina más proteica según la TPCA. Su índice glucémico es 16, muy bajo. Es altamente RECOMENDADO para DM2 por su bajo impacto glucémico y alto aporte proteico.</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>El tarwi es un alimento peruano muy nutritivo y beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, 100g de tarwi contienen aproximadamente:
-- Energía: 343.0 kcal
-- Proteínas: 49.0g
-Estos valores pueden variar ligeramente dependiendo de la variedad y el método de preparación.
-El tarwi es una excelente fuente de proteínas vegetales, lo que lo hace ideal para las personas con diabetes tipo 2. Las proteínas son esenciales para la reparación y construcción de tejidos en el cuerpo, y no elevan los niveles de azúcar en la sangre como lo hacen los carbohidratos.
-Además, el tarwi tiene un Índice Glucémico (IG) muy bajo de 15, lo que significa que su consumo no provoca picos bruscos de glucosa en la sangre. Esto es especialmente importante para las personas con diabetes, que necesitan controlar sus niveles de azúcar en la sangre.
-Por estas razones, el tarwi es un alimento muy recomendable para las personas con diabetes tipo 2. Sin embargo, como con cualquier alimento, es importante consumirlo en cantidades moderadas y dentro de una dieta equilibrada.</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>0.8252</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>El tarwi contiene 249 kcal y 49g de proteínas por 100g según la TPCA CENAN/INS.
+El tarwi es una excelente fuente de proteína para personas con diabetes tipo 2. Tiene un índice glucémico muy bajo (IG=15), lo que significa que no provoca picos significativos en los niveles de glucosa en sangre. Además, su alto contenido de proteínas y fibra ayuda a mantener la saciedad y a regular la absorción de glucosa, lo que es beneficioso para el control de la diabetes. ¡Es una opción nutritiva y saludable!</t>
+        </is>
       </c>
       <c r="H6" t="n">
-        <v>5</v>
+        <v>0.5589</v>
       </c>
       <c r="I6" t="n">
-        <v>3410</v>
+        <v>10</v>
       </c>
       <c r="J6" t="n">
-        <v>307</v>
+        <v>4096</v>
       </c>
       <c r="K6" t="n">
-        <v>12222</v>
+        <v>122</v>
+      </c>
+      <c r="L6" t="n">
+        <v>8211.4</v>
       </c>
     </row>
     <row r="7">
@@ -742,39 +751,38 @@
         <v>115</v>
       </c>
       <c r="D7" t="n">
-        <v>127</v>
+        <v>328</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
           <t>El tarwi cocido y desamargado contiene 115 kcal por 100g según la TPCA. Aporta 15.6g de proteínas, 7.1g de grasas y 9.1g de carbohidratos. Su índice glucémico es 16, muy bajo. RECOMENDADO ampliamente para pacientes con DM2.</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>El tarwi (también conocido como chocho) es un alimento peruano muy nutritivo y beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, 100g de tarwi cocido y desamargado aporta aproximadamente 127 kcal.
-Además, el tarwi tiene un Índice Glucémico (IG) muy bajo de 15, lo que significa que su consumo no provoca picos bruscos en los niveles de azúcar en la sangre. También es una excelente fuente de proteína vegetal (33g por cada 100g) y fibra (18g por cada 100g), nutrientes que ayudan a controlar la glucemia y aportan saciedad.
-Por lo tanto, el tarwi es altamente recomendado para personas con diabetes tipo 2. Recuerda siempre consumirlo en porciones adecuadas y como parte de una dieta equilibrada. 
-🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: [vegetales/ensalada]
-2.° Luego: tarwi (como proteína)
-3.° Al final: [carbohidratos]
-Si tienes alguna otra pregunta sobre la diabetes o la nutrición, no dudes en preguntar.</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>0.8227</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>No tengo el dato exacto en la TPCA sobre las calorías del tarwi cocido y desamargado. Sin embargo, el tarwi (también conocido como chocho o lupino) tiene un Índice Glucémico (IG) de 15, lo que lo clasifica como un alimento de IG muy bajo, recomendado para personas con diabetes. 
+El tarwi es una excelente fuente de proteína vegetal y fibra, lo que ayuda a ralentizar la absorción de glucosa en el organismo. Por lo tanto, sí, un diabético puede incluir tarwi en su dieta, siempre en porciones adecuadas y como parte de una alimentación equilibrada. ¡Es una gran opción!</t>
+        </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>0.5656</v>
       </c>
       <c r="I7" t="n">
-        <v>3394</v>
+        <v>9</v>
       </c>
       <c r="J7" t="n">
-        <v>306</v>
+        <v>4179</v>
       </c>
       <c r="K7" t="n">
-        <v>11380</v>
+        <v>144</v>
+      </c>
+      <c r="L7" t="n">
+        <v>7729.5</v>
       </c>
     </row>
     <row r="8">
@@ -796,28 +804,33 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>La cebada con cáscara contiene 284 kcal por 100g según la TPCA CENAN/INS. Aporta 8.4g de proteínas, 2.0g de grasas y 77.5g de carbohidratos. Tiene 17.3g de fibra dietaria, la más alta entre los cereales evaluados.</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>La cebada con cáscara tiene 284.0 kilocalorías por cada 100 gramos, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>0.8703</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>La cebada con cáscara contiene 284.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H8" t="n">
-        <v>5</v>
+        <v>0.6528</v>
       </c>
       <c r="I8" t="n">
-        <v>3490</v>
+        <v>7</v>
       </c>
       <c r="J8" t="n">
-        <v>57</v>
+        <v>3841</v>
       </c>
       <c r="K8" t="n">
-        <v>15038</v>
+        <v>27</v>
+      </c>
+      <c r="L8" t="n">
+        <v>6678.2</v>
       </c>
     </row>
     <row r="9">
@@ -835,53 +848,37 @@
         <v>284</v>
       </c>
       <c r="D9" t="n">
-        <v>274</v>
+        <v>284</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
           <t>La cebada contiene 284 kcal y 17.3g de fibra por 100g según la TPCA. Su índice glucémico es 28, muy bajo. La alta fibra beta-glucano reduce el pico glucémico postprandial hasta un 30%. RECOMENDADO para DM2.</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>La cebada es un alimento muy nutritivo y beneficioso para personas con diabetes tipo 2. Aquí te presento la información nutricional de diferentes presentaciones de cebada según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS:
-1. **Cebada tostada, harina integral**:
-   - Fibra dietaria: 25.4g por 100g
-   - Calorías: 274.0 kcal por 100g
-   - Índice Glucémico (IG): 60 (moderado)
-2. **Cebada con cáscara**:
-   - Fibra dietaria: 17.3g por 100g
-   - Calorías: 284.0 kcal por 100g
-   - Índice Glucémico (IG): 28 (bajo)
-3. **Cebada para mote, pelada**:
-   - Fibra dietaria: No especificada en la TPCA
-   - Calorías: 328.0 kcal por 100g
-   - Índice Glucémico (IG): 28 (bajo)
-4. **Cebada tostada y molida (chaquepa)**:
-   - Fibra dietaria: No especificada en la TPCA
-   - Calorías: 349.0 kcal por 100g
-   - Índice Glucémico (IG): 28 (bajo)
-5. **Pan de cebada (serrano)**:
-   - Fibra dietaria: No especificada en la TPCA
-   - Calorías: 295.0 kcal por 100g
-   - Índice Glucémico (IG): 28 (bajo)
-La cebada es una excelente fuente de fibra dietaria, lo que ayuda a ralentizar la absorción de glucosa en el cuerpo, contribuyendo a un mejor control de los niveles de azúcar en la sangre. Además, su bajo Índice Glucémico (IG) la hace recomendable para personas con diabetes tipo 2.</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>0.8455</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>La cebada contiene 284 kcal por 100g según la TPCA CENAN/INS. Además, tiene 17.3g de fibra dietaria y un índice glucémico (IG) de 28, lo que la clasifica como un alimento de IG bajo, recomendado para personas con diabetes mellitus tipo 2.</t>
+        </is>
       </c>
       <c r="H9" t="n">
-        <v>5</v>
+        <v>0.6411</v>
       </c>
       <c r="I9" t="n">
-        <v>3461</v>
+        <v>6</v>
       </c>
       <c r="J9" t="n">
-        <v>471</v>
+        <v>3604</v>
       </c>
       <c r="K9" t="n">
-        <v>34712</v>
+        <v>68</v>
+      </c>
+      <c r="L9" t="n">
+        <v>6847.2</v>
       </c>
     </row>
     <row r="10">
@@ -899,44 +896,39 @@
         <v>284</v>
       </c>
       <c r="D10" t="n">
-        <v>328</v>
+        <v>284</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
           <t>La cebada tiene 284 kcal/100g con IG 28, mientras el arroz pilado tiene 115 kcal cocido con IG 73. La cebada es SUPERIOR para DM2 por su menor índice glucémico y mayor fibra (17.3g vs 0.3g). Sustituir arroz por cebada reduce el pico glucémico postprandial significativamente.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>La cebada y el arroz son ambos granos que pueden formar parte de una dieta saludable para personas con diabetes tipo 2, pero tienen diferencias nutricionales significativas que pueden afectar su impacto en los niveles de azúcar en sangre.
-🌾 **Cebada (para mote, pelada)**:
-- Energía: 328.0 kcal por 100g
-- Índice Glucémico (IG): 28 (bajo)
-- Carbohidratos totales: 73.3g por 100g
-🍚 **Arroz blanco (cocido)**:
-- Energía: aproximadamente 130 kcal por 100g
-- Índice Glucémico (IG): alrededor de 73 (alto)
-- Carbohidratos totales: alrededor de 28g por 100g
-Aunque la cebada tiene más calorías y carbohidratos que el arroz blanco por 100g, su IG es significativamente más bajo. Esto significa que la cebada provoca un aumento más lento y gradual de la glucosa en sangre en comparación con el arroz blanco, lo cual es beneficioso para las personas con diabetes.
-Además, la cebada es rica en fibra dietaria, que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo y a mantener la sensación de saciedad por más tiempo.
-Por lo tanto, para un paciente con diabetes tipo 2, la cebada puede ser una opción más saludable que el arroz blanco, siempre y cuando se tenga en cuenta el tamaño de la porción para no exceder la ingesta diaria recomendada de carbohidratos.
-Recuerda siempre consultar a tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>0.8354</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>La cebada contiene 284 kcal por 100g según la TPCA CENAN/INS, mientras que el arroz blanco contiene aproximadamente 130 kcal por 100g. 
+En cuanto a cuál es mejor para un diabético, la cebada es una mejor opción. Tiene un Índice Glucémico (IG) de 28, lo que la clasifica como un alimento de IG bajo, mientras que el arroz blanco tiene un IG más alto (alrededor de 70), lo que puede provocar un aumento más rápido de la glucosa en sangre. 
+La cebada también es rica en fibra (17.3g por 100g), lo que ayuda a ralentizar la absorción de glucosa y mejora el control de la glucemia. Por lo tanto, te recomendaría optar por la cebada en lugar del arroz.</t>
+        </is>
       </c>
       <c r="H10" t="n">
+        <v>0.5647</v>
+      </c>
+      <c r="I10" t="n">
         <v>5</v>
       </c>
-      <c r="I10" t="n">
-        <v>3431</v>
-      </c>
       <c r="J10" t="n">
-        <v>406</v>
+        <v>3333</v>
       </c>
       <c r="K10" t="n">
-        <v>10483</v>
+        <v>173</v>
+      </c>
+      <c r="L10" t="n">
+        <v>8125.9</v>
       </c>
     </row>
     <row r="11">
@@ -954,32 +946,37 @@
         <v>333</v>
       </c>
       <c r="D11" t="n">
-        <v>333</v>
+        <v>380</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>La avena en hojuela cruda contiene 333 kcal por 100g según la TPCA CENAN/INS. Aporta 13.3g de proteínas, 4.0g de grasas y 72.2g de carbohidratos. Tiene 10.6g de fibra dietaria (beta-glucano).</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>La avena en hojuela cruda tiene 333.0 kcal por cada 100 gramos, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>0.8563</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>La avena en hojuela cruda contiene 333.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H11" t="n">
-        <v>5</v>
+        <v>0.5674</v>
       </c>
       <c r="I11" t="n">
-        <v>3618</v>
+        <v>8</v>
       </c>
       <c r="J11" t="n">
-        <v>56</v>
+        <v>4263</v>
       </c>
       <c r="K11" t="n">
-        <v>16163</v>
+        <v>29</v>
+      </c>
+      <c r="L11" t="n">
+        <v>8631.299999999999</v>
       </c>
     </row>
     <row r="12">
@@ -997,43 +994,38 @@
         <v>333</v>
       </c>
       <c r="D12" t="n">
-        <v>54</v>
+        <v>380</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
           <t>La avena contiene 333 kcal y 10.6g de fibra beta-glucano por 100g según la TPCA. El beta-glucano forma un gel viscoso en el intestino que retarda la absorción de glucosa. RECOMENDADO para DM2 con IG 55. Reduce la hemoglobina glicosilada HbA1c.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>La avena es un alimento muy beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, existen diferentes presentaciones de avena, cada una con su propia composición nutricional. Aquí te presento dos ejemplos:
-1. **Avena, hojuela cocida**:
-   - Energía: 54.0 kcal por 100g
-   - Fibra dietaria: No especificada, pero la avena generalmente es alta en fibra.
-2. **Avena con chía, hojuela precocida**:
-   - Energía: 381.0 kcal por 100g
-   - Fibra dietaria: 13.0g por 100g
-La avena es especialmente beneficiosa para las personas con diabetes por varias razones:
-- **Índice glucémico bajo (IG=55)**: Esto significa que los carbohidratos en la avena se absorben lentamente, lo que ayuda a evitar los picos de azúcar en la sangre que pueden ocurrir después de comer alimentos con un IG alto.
-- **Alta en fibra**: La fibra ayuda a ralentizar la absorción de azúcar en la sangre, lo que puede ayudar a controlar los niveles de glucosa.
-- **Contiene beta-glucanos**: Este es un tipo de fibra soluble que puede mejorar la sensibilidad a la insulina y ayudar a mantener los niveles de azúcar en la sangre bajo control.
-Recuerda siempre consumir la avena en porciones adecuadas y preferiblemente sin azúcares añadidos para mantener un buen control de tu diabetes. Consulta con tu médico o nutricionista para obtener recomendaciones personalizadas.</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>0.8401</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>La avena contiene 380.0 kcal por 100g según la TPCA CENAN/INS y tiene 10.6g de fibra por cada 100g.
+La avena es beneficiosa para personas con diabetes porque tiene un Índice Glucémico (IG) de 55, lo que significa que su impacto en los niveles de glucosa en sangre es moderado. La fibra presente en la avena ayuda a ralentizar la absorción de glucosa, lo que puede contribuir a mantener niveles de azúcar en sangre más estables. Además, la fibra favorece la saciedad, lo que puede ayudar a controlar el apetito y el peso. ¡Incluir avena en tu dieta puede ser una excelente decisión!</t>
+        </is>
       </c>
       <c r="H12" t="n">
-        <v>5</v>
+        <v>0.5572</v>
       </c>
       <c r="I12" t="n">
-        <v>3563</v>
+        <v>7</v>
       </c>
       <c r="J12" t="n">
-        <v>411</v>
+        <v>3976</v>
       </c>
       <c r="K12" t="n">
-        <v>30358</v>
+        <v>151</v>
+      </c>
+      <c r="L12" t="n">
+        <v>8213.299999999999</v>
       </c>
     </row>
     <row r="13">
@@ -1055,34 +1047,35 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
           <t>La avena envasada contiene 380 kcal por 100g según la TPCA. Aporta 13.7g de proteínas, 4.7g de grasas y 71.3g de carbohidratos. IG 55, RECOMENDADO para desayuno DM2. Combinar con tarwi o kiwicha mejora el perfil proteico.</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>La avena envasada tiene 380.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Y sí, la avena envasada es una excelente opción de desayuno para una persona con diabetes tipo 2. Aquí te explico por qué:
-1. **Índice Glucémico (IG) bajo (55)**: Los alimentos con IG bajo se digieren y absorben lentamente, lo que produce un aumento gradual y más manejable de los niveles de azúcar en la sangre.
-2. **Rica en fibra**: La avena es una fuente de fibra dietética, que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo, evitando picos bruscos de azúcar en la sangre.
-3. **Proteínas**: Con 13.7g de proteínas por cada 100g, la avena puede ayudar a mantener la sensación de saciedad, lo que es beneficioso para el control del peso.
-Recuerda seguir la secuencia alimentaria recomendada: empieza con una porción de frutas o verduras, luego consume la avena y finalmente cualquier otro alimento con carbohidratos. Esto puede ayudar a reducir el pico glucémico posprandial.
-Además, ten en cuenta que la cantidad de avena que consumas debe ajustarse a tus necesidades individuales de carbohidratos y calorías. Consulta con tu médico o nutricionista para determinar la porción adecuada para ti.</t>
-        </is>
-      </c>
-      <c r="G13" t="n">
-        <v>0.8339</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>La avena envasada contiene 380.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, la avena es una buena opción de desayuno para personas con diabetes tipo 2. Tiene un Índice Glucémico (IG) de 55, lo que se considera bajo, y aporta una buena cantidad de fibra (que ayuda a regular la glucosa en sangre) y proteínas. Además, su consumo puede proporcionar una sensación de saciedad, lo que puede ayudar a controlar el apetito a lo largo del día. 
+Recuerda siempre combinarla con otros alimentos saludables y seguir el orden de consumo recomendado para maximizar los beneficios. ¡Excelente decisión al considerar la avena!</t>
+        </is>
       </c>
       <c r="H13" t="n">
-        <v>5</v>
+        <v>0.5749</v>
       </c>
       <c r="I13" t="n">
-        <v>3537</v>
+        <v>6</v>
       </c>
       <c r="J13" t="n">
-        <v>374</v>
+        <v>3690</v>
       </c>
       <c r="K13" t="n">
-        <v>18505</v>
+        <v>147</v>
+      </c>
+      <c r="L13" t="n">
+        <v>10165.9</v>
       </c>
     </row>
     <row r="14">
@@ -1100,32 +1093,37 @@
         <v>353</v>
       </c>
       <c r="D14" t="n">
-        <v>343</v>
+        <v>353</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
           <t>La lenteja cruda contiene 353 kcal por 100g según la TPCA CENAN/INS. Aporta 25.8g de proteínas, 1.8g de grasas y 60.1g de carbohidratos. Tiene 11.4g de fibra dietaria. IG 29, muy bajo.</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, 100 gramos de lentejas crudas contienen aproximadamente 343.0 kcal. Ten en cuenta que este valor puede variar ligeramente dependiendo de la variedad específica de lenteja y su contenido de agua. Recuerda que las lentejas son una excelente fuente de proteínas y fibra, lo que las hace una buena opción para las personas con diabetes tipo 2.</t>
-        </is>
-      </c>
-      <c r="G14" t="n">
-        <v>0.8468</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>La lenteja cruda contiene 353.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H14" t="n">
-        <v>5</v>
+        <v>0.5872000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>3490</v>
+        <v>8</v>
       </c>
       <c r="J14" t="n">
-        <v>112</v>
+        <v>3580</v>
       </c>
       <c r="K14" t="n">
-        <v>9136</v>
+        <v>25</v>
+      </c>
+      <c r="L14" t="n">
+        <v>6186.7</v>
       </c>
     </row>
     <row r="15">
@@ -1143,35 +1141,38 @@
         <v>114</v>
       </c>
       <c r="D15" t="n">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
           <t>La lenteja cocida contiene 114 kcal por 100g según la TPCA. Aporta 8.4g de proteínas, 0.6g de grasas y 19.5g de carbohidratos. IG 29, muy bajo. RECOMENDADO 3-4 veces por semana para DM2. Excelente fuente de proteína vegetal y hierro.</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>La lenteja cocida es un alimento muy nutritivo y beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, por cada 100g de lentejas cocidas, se obtienen aproximadamente 116 kcal. 
-Las lentejas son una excelente fuente de fibra dietética, que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo y a controlar los niveles de azúcar en la sangre. Además, tienen un Índice Glucémico (IG) bajo, lo que significa que no elevan rápidamente los niveles de azúcar en la sangre.
-En cuanto a la frecuencia de consumo, las lentejas pueden ser incluidas en la dieta de un diabético varias veces a la semana, siempre y cuando se mantenga una porción adecuada y se combine con otros alimentos de bajo IG. Recuerda que el control de las porciones es clave para mantener un equilibrio nutricional y evitar picos de glucosa en la sangre.
-Como siempre, te recomiendo que consultes con tu médico o un dietista registrado antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>0.8159</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>La lenteja cocida contiene 114.0 kcal por 100g según la TPCA CENAN/INS. 
+Para un paciente con diabetes tipo 2, las lentejas son una excelente opción debido a su bajo índice glucémico (IG=29) y su alto contenido de fibra. Puedes incluir lentejas en tu dieta de 2 a 3 veces por semana, siempre considerando la porción adecuada y combinándolas con verduras y proteínas para mantener un buen control de la glucosa. ¡Recuerda siempre consultar con tu médico o nutricionista para personalizar tu plan alimenticio!</t>
+        </is>
       </c>
       <c r="H15" t="n">
-        <v>5</v>
+        <v>0.498</v>
       </c>
       <c r="I15" t="n">
-        <v>3408</v>
+        <v>6</v>
       </c>
       <c r="J15" t="n">
-        <v>278</v>
+        <v>3394</v>
       </c>
       <c r="K15" t="n">
-        <v>25798</v>
+        <v>122</v>
+      </c>
+      <c r="L15" t="n">
+        <v>7456.3</v>
       </c>
     </row>
     <row r="16">
@@ -1189,39 +1190,39 @@
         <v>353</v>
       </c>
       <c r="D16" t="n">
-        <v>116</v>
+        <v>353</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
           <t>La lenteja cruda aporta 353 kcal y 25.8g de proteínas por 100g según la TPCA. Contiene 7.6mg de hierro y 11.4g de fibra. Su IG de 29 la hace ideal para DM2. RECOMENDADO como sustituto de la carne roja en la dieta del diabético.</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, las lentejas cocidas tienen la siguiente composición por 100g de porción comestible:
-- Energía: 116.0 kcal
-- Proteínas: 9.0g
-- Hierro: 3.3mg
-Además, las lentejas tienen un Índice Glucémico (IG) de 30, lo que las clasifica como un alimento de IG bajo, recomendado para pacientes con diabetes mellitus tipo 2.
-Las lentejas son una excelente opción para las personas con diabetes. Son ricas en proteínas y fibra dietética, lo que ayuda a controlar los niveles de azúcar en la sangre al ralentizar la absorción de glucosa. Además, su contenido de hierro contribuye a la prevención de la anemia.
-Recuerda que es importante consumir las lentejas en porciones adecuadas y en combinación con otros alimentos de IG bajo para mantener un control óptimo de la glucemia. 
-Fuente: Tabla Peruana de Composición de Alimentos (TPCA) 2025, CENAN/INS, MINSA Perú.</t>
-        </is>
-      </c>
-      <c r="G16" t="n">
-        <v>0.8133</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>La lenteja cruda contiene 353.0 kcal por 100g según la TPCA CENAN/INS, y aporta 25.8g de proteínas. 
+Además, las lentejas son una buena fuente de hierro, lo que puede ser beneficioso para diabéticos, ya que el hierro es esencial para la producción de glóbulos rojos y el transporte de oxígeno en el cuerpo. Sin embargo, es importante consumirlas en combinación con alimentos ricos en vitamina C para mejorar la absorción del hierro. 
+Recuerda siempre consultar con tu médico o nutricionista sobre tus necesidades específicas.</t>
+        </is>
       </c>
       <c r="H16" t="n">
-        <v>5</v>
+        <v>0.5101</v>
       </c>
       <c r="I16" t="n">
-        <v>3428</v>
+        <v>7</v>
       </c>
       <c r="J16" t="n">
-        <v>275</v>
+        <v>3445</v>
       </c>
       <c r="K16" t="n">
-        <v>19299</v>
+        <v>123</v>
+      </c>
+      <c r="L16" t="n">
+        <v>7918.8</v>
       </c>
     </row>
     <row r="17">
@@ -1238,31 +1239,38 @@
       <c r="C17" t="n">
         <v>105</v>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>105</v>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
           <t>El camote amarillo crudo contiene 105 kcal por 100g según la TPCA CENAN/INS. Aporta 1.6g de proteínas, 0.3g de grasas y 24.3g de carbohidratos. Tiene 3.0g de fibra dietaria.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>El camote amarillo crudo no está en mi base de datos de la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS. Sin embargo, puedo decirte que, en general, el camote crudo tiene alrededor de 86 calorías por 100 gramos. Este valor puede variar un poco dependiendo del tipo específico de camote. Recuerda que el camote tiene un Índice Glucémico medio, por lo que es recomendable consumirlo con moderación si tienes diabetes tipo 2.</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>0.829</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>El camote amarillo crudo contiene 105.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H17" t="n">
-        <v>5</v>
+        <v>0.5795</v>
       </c>
       <c r="I17" t="n">
-        <v>3547</v>
+        <v>8</v>
       </c>
       <c r="J17" t="n">
-        <v>125</v>
+        <v>4070</v>
       </c>
       <c r="K17" t="n">
-        <v>12388</v>
+        <v>26</v>
+      </c>
+      <c r="L17" t="n">
+        <v>6532.2</v>
       </c>
     </row>
     <row r="18">
@@ -1280,35 +1288,39 @@
         <v>105</v>
       </c>
       <c r="D18" t="n">
-        <v>483</v>
+        <v>105</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
           <t>El camote tiene 105 kcal/100g con IG 54, mejor que la papa blanca (97 kcal, IG 70). El camote es RECOMENDADO para DM2 por su menor IG y mayor contenido de betacarotenos. La papa blanca es LIMITAR por su alto IG que eleva la glucosa rápidamente.</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>El camote, en su versión de hojuela frita en aceite vegetal y endulzado, tiene 483.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS. Sin embargo, este tipo de preparación no es la más saludable para un paciente con diabetes tipo 2 debido a su alto contenido de grasas y carbohidratos.
-Comparando el camote con la papa, ambos son tubérculos ricos en carbohidratos. Sin embargo, el camote tiene un Índice Glucémico (IG) generalmente más bajo que la papa, lo que significa que sus carbohidratos se absorben más lentamente, causando un aumento más gradual de los niveles de azúcar en la sangre. Esto puede ser beneficioso para las personas con diabetes tipo 2.
-Además, el camote es rico en fibra dietaria, que también ayuda a regular los niveles de azúcar en la sangre. Por lo tanto, en general, el camote puede ser una opción más saludable que la papa para las personas con diabetes tipo 2, siempre y cuando se prepare de manera saludable (hervido o al horno, no frito) y se consuma en porciones moderadas.
-Recuerda siempre consultar con tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>0.8143</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>El camote amarillo contiene 105.0 kcal por 100g según la TPCA CENAN/INS. 
+En cuanto a la comparación con la papa, el camote es generalmente mejor para un paciente con diabetes tipo 2. Esto se debe a que el camote tiene un Índice Glucémico (IG) de 54, que es considerado bajo, mientras que la papa tiene un IG más alto, lo que puede provocar un aumento más rápido de la glucosa en sangre. Además, el camote aporta más fibra (3.0g por 100g) que la papa, lo que ayuda a mejorar el control glucémico. 
+Recuerda siempre consultar con tu médico o nutricionista antes de hacer cambios significativos en tu dieta. ¡Cada elección cuenta!</t>
+        </is>
       </c>
       <c r="H18" t="n">
+        <v>0.5741000000000001</v>
+      </c>
+      <c r="I18" t="n">
         <v>5</v>
       </c>
-      <c r="I18" t="n">
-        <v>3451</v>
-      </c>
       <c r="J18" t="n">
-        <v>324</v>
+        <v>3286</v>
       </c>
       <c r="K18" t="n">
-        <v>27134</v>
+        <v>161</v>
+      </c>
+      <c r="L18" t="n">
+        <v>7929.9</v>
       </c>
     </row>
     <row r="19">
@@ -1326,41 +1338,43 @@
         <v>105</v>
       </c>
       <c r="D19" t="n">
-        <v>483</v>
+        <v>105</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
           <t>El camote amarillo contiene 105 kcal y es rico en betacarotenos (vitamina A precursora) según la TPCA. Aporta 3.0g de fibra. Su IG de 54 es moderado. RECOMENDADO para DM2 en porciones de 100-150g. Los betacarotenos tienen acción antioxidante.</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>El camote, en su versión de hojuela frita en aceite vegetal y endulzado, aporta 483.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-En cuanto a los micronutrientes, el camote proporciona:
-- Calcio: 14.0mg
-- Hierro: 3.11mg
-- Zinc: 0.31mg
-- Fósforo: 120.0mg
-- Sodio: 206.0mg
-- Potasio: 72.0mg
-Es importante mencionar que esta versión del camote tiene un Índice Glucémico (IG) de 61, lo que es considerado medio. Esto significa que debe consumirse con moderación en personas con diabetes tipo 2 para evitar picos en los niveles de glucosa en sangre. Además, contiene 7.2g de fibra dietaria, que ayuda a ralentizar la absorción de glucosa y a mantener la sensación de saciedad.
-Recuerda que es esencial mantener una dieta equilibrada y variada para asegurar la ingesta adecuada de todos los nutrientes necesarios. Consulta con tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>0.8264</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>El camote amarillo crudo contiene 105.0 kcal por 100g según la TPCA CENAN/INS. 
+En cuanto a los micronutrientes que aporta, el camote es una excelente fuente de nutrientes beneficiosos para personas con diabetes, incluyendo:
+- **Fibra**: 3.0g, que ayuda a regular la glucosa en sangre.
+- **Vitamina A**: importante para la salud ocular y el sistema inmunológico.
+- **Vitamina C**:  proporciona antioxidantes que ayudan a combatir el estrés oxidativo.
+- **Potasio**:  ayuda a mantener la presión arterial y la función cardíaca.
+Además, su índice glucémico es de 54, lo que lo clasifica como un alimento de IG bajo, recomendado para personas con diabetes. Esto significa que su consumo no provoca picos significativos en los niveles de glucosa en sangre. ¡Es una excelente opción para incluir en tu dieta!</t>
+        </is>
       </c>
       <c r="H19" t="n">
-        <v>5</v>
+        <v>0.5521</v>
       </c>
       <c r="I19" t="n">
-        <v>3423</v>
+        <v>10</v>
       </c>
       <c r="J19" t="n">
-        <v>301</v>
+        <v>4613</v>
       </c>
       <c r="K19" t="n">
-        <v>18865</v>
+        <v>196</v>
+      </c>
+      <c r="L19" t="n">
+        <v>9020.5</v>
       </c>
     </row>
     <row r="20">
@@ -1382,28 +1396,33 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>El aguaymanto contiene 53 kcal por 100g según la TPCA CENAN/INS 2025. Aporta 1.9g de proteínas, 0.7g de grasas y 11.2g de carbohidratos. Tiene 2.0g de fibra y alto contenido de vitamina C y withanólidos.</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>El aguaymanto tiene 51.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>0.8485</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>El aguaymanto contiene 51.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H20" t="n">
-        <v>5</v>
+        <v>0.6018</v>
       </c>
       <c r="I20" t="n">
-        <v>3505</v>
+        <v>10</v>
       </c>
       <c r="J20" t="n">
-        <v>57</v>
+        <v>4627</v>
       </c>
       <c r="K20" t="n">
-        <v>10389</v>
+        <v>25</v>
+      </c>
+      <c r="L20" t="n">
+        <v>6884.6</v>
       </c>
     </row>
     <row r="21">
@@ -1425,31 +1444,35 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
           <t>El aguaymanto contiene 53 kcal por 100g. Sus withanólidos tienen efecto hipoglucemiante demostrado en estudios. IG 25, muy bajo. Aporta vitamina C y antioxidantes. RECOMENDADO para DM2 como fruta de consumo regular para control de la glucosa.</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>El aguaymanto es una fruta peruana con un contenido calórico de 51.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Además, el aguaymanto es una excelente fuente de vitamina C, con 43.3mg por cada 100g. La vitamina C es un poderoso antioxidante que ayuda a proteger las células del cuerpo contra los daños causados por los radicales libres. En personas con diabetes, el estrés oxidativo puede aumentar debido a los niveles altos de glucosa en sangre, por lo que consumir alimentos ricos en antioxidantes como el aguaymanto puede ser beneficioso.
-Además, el aguaymanto tiene un Índice Glucémico (IG) de 25, que es considerado bajo. Los alimentos con un IG bajo liberan glucosa lentamente y de manera más estable en el torrente sanguíneo, lo que puede ayudar a controlar los niveles de azúcar en sangre en personas con diabetes.
-Recuerda que, aunque el aguaymanto es beneficioso, debe consumirse dentro de una dieta equilibrada y variada. Siempre es recomendable consultar a un profesional de la salud antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G21" t="n">
-        <v>0.8253</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>El aguaymanto contiene 51.0 kcal por 100g según la TPCA CENAN/INS. 
+En cuanto a sus propiedades antioxidantes, el aguaymanto es rico en vitamina C y otros compuestos fenólicos que ayudan a combatir el estrés oxidativo. Esto es especialmente beneficioso para personas con diabetes, ya que el estrés oxidativo puede contribuir a las complicaciones de la enfermedad. Además, su bajo índice glucémico (IG=25) lo convierte en una opción segura y saludable para incluir en la dieta de pacientes con diabetes mellitus tipo 2. 
+¡Incluir aguaymanto en tu alimentación puede ser una excelente decisión! 🍇</t>
+        </is>
       </c>
       <c r="H21" t="n">
-        <v>5</v>
+        <v>0.5528999999999999</v>
       </c>
       <c r="I21" t="n">
-        <v>3552</v>
+        <v>10</v>
       </c>
       <c r="J21" t="n">
-        <v>311</v>
+        <v>4735</v>
       </c>
       <c r="K21" t="n">
-        <v>23383</v>
+        <v>139</v>
+      </c>
+      <c r="L21" t="n">
+        <v>6591.3</v>
       </c>
     </row>
     <row r="22">
@@ -1471,34 +1494,35 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
           <t>El aguaymanto aporta 53 kcal y alto contenido de vitamina C según la TPCA. Con IG 25 es mejor opción que el mango (IG 51) o la chirimoya (IG 35) para DM2. RECOMENDADO como la fruta andina más adecuada para control glucémico en DM2.</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>El aguaymanto es una excelente opción para personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, cada 100g de aguaymanto contiene:
-- Energía: 51.0 kcal
-- Vitamina C: 43.3mg
-Además, tiene un Índice Glucémico (IG) de 25, que es considerado bajo. Esto significa que su consumo no provoca un aumento brusco en los niveles de glucosa en la sangre.
-Comparado con otras frutas, el aguaymanto tiene ventajas para personas con diabetes. Por ejemplo, su contenido de fibra dietaria (4.9g por 100g) ayuda a ralentizar la absorción de glucosa, lo que contribuye a un mejor control de la glucemia. Además, su contenido de vitamina C es bastante alto, lo que es beneficioso para el sistema inmunológico.
-Recuerda que es importante consumir una variedad de frutas para obtener un amplio espectro de nutrientes. Otras frutas con IG bajo recomendadas para diabéticos son la granadilla, el mango ciruelo o taperibá, el aguaje y la guayaba amarilla. 
-Siempre es recomendable consultar con tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G22" t="n">
-        <v>0.8212</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>El aguaymanto contiene 51.0 kcal por 100g según la TPCA CENAN/INS y tiene 43.3 mg de vitamina C por la misma cantidad.
+En cuanto a su idoneidad para personas con diabetes, el aguaymanto tiene un Índice Glucémico (IG) de 25, lo que lo clasifica como un alimento de IG bajo, recomendado para diabéticos. Esto significa que su consumo no provoca picos significativos en los niveles de glucosa en sangre, en comparación con frutas de IG más alto.
+Además, el aguaymanto es rico en fibra (4.9g por 100g), lo que también ayuda a regular la glucosa. En general, es una excelente opción entre las frutas para personas con diabetes, pero siempre es bueno variar el consumo de frutas y verduras para obtener un rango completo de nutrientes.</t>
+        </is>
       </c>
       <c r="H22" t="n">
-        <v>5</v>
+        <v>0.5659999999999999</v>
       </c>
       <c r="I22" t="n">
-        <v>3561</v>
+        <v>10</v>
       </c>
       <c r="J22" t="n">
-        <v>313</v>
+        <v>4700</v>
       </c>
       <c r="K22" t="n">
-        <v>20142</v>
+        <v>182</v>
+      </c>
+      <c r="L22" t="n">
+        <v>10175.8</v>
       </c>
     </row>
     <row r="23">
@@ -1520,28 +1544,33 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
           <t>La palta o aguacate contiene 177 kcal por 100g según la TPCA CENAN/INS. Aporta 2.0g de proteínas, 17.0g de grasas (principalmente monoinsaturadas) y 6.3g de carbohidratos. Tiene 6.7g de fibra dietaria. IG 15, muy bajo.</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>La palta o aguacate tiene 130.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>0.8508</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>La palta contiene 130.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H23" t="n">
-        <v>5</v>
+        <v>0.6405</v>
       </c>
       <c r="I23" t="n">
-        <v>3425</v>
+        <v>6</v>
       </c>
       <c r="J23" t="n">
-        <v>59</v>
+        <v>3464</v>
       </c>
       <c r="K23" t="n">
-        <v>14801</v>
+        <v>23</v>
+      </c>
+      <c r="L23" t="n">
+        <v>6185.7</v>
       </c>
     </row>
     <row r="24">
@@ -1559,37 +1588,39 @@
         <v>177</v>
       </c>
       <c r="D24" t="n">
-        <v>130</v>
+        <v>166</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
           <t>La palta tiene 177 kcal y 17.0g de grasas monoinsaturadas (ácido oleico) por 100g según la TPCA. Las grasas monoinsaturadas mejoran la sensibilidad a la insulina y reducen el colesterol LDL. IG 15. RECOMENDADO para DM2 en porciones de 1/4 a 1/2 palta diaria.</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>La palta es un alimento muy nutritivo y beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, 100g de palta contienen:
-- Palta común: 130.0 kcal y 12.5g de grasas.
-- Palta Hass: 204.0 kcal y 23.5g de grasas.
-Las grasas presentes en la palta son mayormente grasas monoinsaturadas y poliinsaturadas, conocidas como "grasas buenas". Estas grasas ayudan a reducir los niveles de colesterol LDL (malo) y aumentar el colesterol HDL (bueno), lo que es beneficioso para la salud del corazón. Además, la palta tiene un Índice Glucémico (IG) muy bajo de 15, lo que significa que su consumo no provoca picos bruscos en los niveles de azúcar en sangre.
-Recuerda que, aunque la palta es saludable, es un alimento de alta densidad calórica debido a su contenido de grasa, por lo que su consumo debe ser moderado. Una porción recomendada podría ser 1/4 o 1/2 palta, dependiendo del resto de tu dieta y tus necesidades calóricas.
-Siempre es recomendable consultar a tu médico o nutricionista antes de hacer cambios importantes en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>0.8274</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>La palta contiene 130.0 kcal por 100g según la TPCA CENAN/INS. En cuanto a las grasas, tiene 12.5g por cada 100g.
+Las grasas de la palta son principalmente grasas saludables, como los ácidos grasos monoinsaturados, que son beneficiosos para la salud cardiovascular. Estas grasas pueden ayudar a mejorar los niveles de colesterol y son recomendadas para personas con diabetes, ya que no afectan de manera negativa los niveles de glucosa en sangre. Además, la palta tiene un índice glucémico muy bajo (IG=15), lo que la hace apta para pacientes con diabetes mellitus tipo 2. 
+Incluir palta en tu dieta puede ser una excelente opción, siempre en porciones adecuadas. ¡Recuerda disfrutarla de manera equilibrada! 🥑</t>
+        </is>
       </c>
       <c r="H24" t="n">
-        <v>5</v>
+        <v>0.5422</v>
       </c>
       <c r="I24" t="n">
-        <v>3590</v>
+        <v>7</v>
       </c>
       <c r="J24" t="n">
-        <v>330</v>
+        <v>3800</v>
       </c>
       <c r="K24" t="n">
-        <v>28849</v>
+        <v>173</v>
+      </c>
+      <c r="L24" t="n">
+        <v>9438.1</v>
       </c>
     </row>
     <row r="25">
@@ -1611,34 +1642,35 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
           <t>Sí, la palta es RECOMENDADA para DM2. Contiene 177 kcal con IG 15, muy bajo. Sus grasas monoinsaturadas (17g/100g) y fibra (6.7g) no elevan la glucosa. Mejoran la sensibilidad a la insulina. Consumo recomendado: 1/4 palta (50g) por porción.</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>¡Claro que sí! La palta es un alimento recomendado para pacientes con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, la palta tiene un Índice Glucémico (IG) muy bajo de 15, lo que significa que su consumo no provoca picos bruscos en los niveles de azúcar en la sangre.
-En cuanto a las calorías, depende del tipo de palta:
-- Palta común: 130.0 kcal por 100g.
-- Palta Hass: 204.0 kcal por 100g.
-- Palta dedo o cocktail: 166.0 kcal por 100g.
-- Palta "fuerte": 104.0 kcal por 100g.
-Además, la palta es rica en grasas saludables, fibra y varios nutrientes esenciales, lo que la hace una excelente opción para una dieta balanceada y saludable. Recuerda siempre consumirla con moderación debido a su contenido calórico.</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>0.8306</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>¡Claro que sí! La palta es una excelente opción para pacientes con diabetes tipo 2. Contiene grasas saludables y tiene un índice glucémico muy bajo, lo que la hace segura para incluir en la dieta.
+La palta contiene 130.0 kcal por 100g según la TPCA CENAN/INS. Además, su índice glucémico es de 15, lo que significa que no provoca picos de glucosa en sangre. 
+Recuerda siempre consultar con tu médico o nutricionista sobre las porciones adecuadas para ti. ¡Excelente decisión al considerar la palta en tu alimentación! 🥑</t>
+        </is>
       </c>
       <c r="H25" t="n">
-        <v>5</v>
+        <v>0.5528</v>
       </c>
       <c r="I25" t="n">
-        <v>3596</v>
+        <v>8</v>
       </c>
       <c r="J25" t="n">
-        <v>237</v>
+        <v>4291</v>
       </c>
       <c r="K25" t="n">
-        <v>13621</v>
+        <v>129</v>
+      </c>
+      <c r="L25" t="n">
+        <v>8384.4</v>
       </c>
     </row>
     <row r="26">
@@ -1656,32 +1688,37 @@
         <v>381</v>
       </c>
       <c r="D26" t="n">
-        <v>381</v>
+        <v>327</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
           <t>La cañihua variedad amarilla contiene 381 kcal por 100g según la TPCA CENAN/INS. Aporta 15.7g de proteínas, 7.5g de grasas y 62.5g de carbohidratos. IG 45, bajo. RECOMENDADO para pacientes con diabetes tipo 2.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>La cañihua amarilla tiene 381.0 kilocalorías por cada 100 gramos de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.</t>
-        </is>
-      </c>
-      <c r="G26" t="n">
-        <v>0.8531</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>La cañihua amarilla contiene 381.0 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H26" t="n">
-        <v>5</v>
+        <v>0.6356000000000001</v>
       </c>
       <c r="I26" t="n">
-        <v>3378</v>
+        <v>6</v>
       </c>
       <c r="J26" t="n">
-        <v>63</v>
+        <v>3547</v>
       </c>
       <c r="K26" t="n">
-        <v>17245</v>
+        <v>27</v>
+      </c>
+      <c r="L26" t="n">
+        <v>6398.8</v>
       </c>
     </row>
     <row r="27">
@@ -1699,35 +1736,44 @@
         <v>381</v>
       </c>
       <c r="D27" t="n">
-        <v>355</v>
+        <v>382</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
           <t>La cañihua contiene 381 kcal por 100g, con 15.7g proteínas (mayor que quinua 13.6g). Rica en hierro y calcio según la TPCA. IG 45, menor que quinua (IG 53). RECOMENDADO para DM2. Es el grano andino menos conocido pero con mayor densidad nutricional.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>La cañihua es un alimento muy nutritivo y beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, la cañihua parda proporciona 355.0 kcal por cada 100g de porción comestible. Además, es rica en minerales como calcio (171.0mg), hierro (15.0mg) y fósforo (496.0mg). 
-Por otro lado, la quinua también es un excelente alimento para las personas con diabetes tipo 2. Según la TPCA, las hojuelas de quinua proporcionan 376.0 kcal por cada 100g de porción comestible. También es rica en calcio (114.0mg), hierro (5.46mg) y fósforo (60.0mg).
-En términos de Índice Glucémico (IG), ambos alimentos son recomendables para personas con diabetes tipo 2. La cañihua tiene un IG de 45, mientras que la quinua tiene un IG de 53. Ambos valores son considerados bajos, lo que significa que estos alimentos no provocan un aumento rápido de los niveles de azúcar en la sangre.
-En conclusión, tanto la cañihua como la quinua son excelentes opciones para las personas con diabetes tipo 2. Ambos alimentos son ricos en nutrientes y tienen un IG bajo. Sin embargo, la cañihua tiene un poco más de proteínas y fibra que la quinua, lo que puede ayudar a controlar los niveles de azúcar en la sangre de una manera más efectiva. Como siempre, es importante recordar que la moderación es clave y que estos alimentos deben ser parte de una dieta equilibrada y saludable.</t>
-        </is>
-      </c>
-      <c r="G27" t="n">
-        <v>0.8459</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>La cañihua contiene 382 kcal por 100g según la TPCA CENAN/INS. En cuanto a minerales, por cada 100g, la cañihua aporta:
+- Calcio: 87-182 mg (dependiendo de la variedad)
+- Hierro: 10.8-17.07 mg
+- Zinc: 4.55-5.68 mg
+- Fósforo: 320-496 mg
+Respecto a si es mejor que la quinua para diabéticos, ambas son opciones saludables, pero la cañihua tiene un Índice Glucémico (IG) de 45, que es considerado bajo y recomendado para personas con diabetes. La quinua, por su parte, tiene un IG de 53, que es un poco más alto. 
+Sin embargo, la elección entre cañihua y quinua también puede depender de otros factores como el contenido de proteínas, fibra y preferencias personales. La cañihua tiene un contenido de proteínas similar y un poco más de fibra en algunas variedades, lo que puede ser beneficioso para el control de la glucosa. 
+En resumen, la cañihua puede ser una excelente opción para diabéticos, pero ambas pueden ser incluidas en una dieta equilibrada. ¡Cada elección cuenta!</t>
+        </is>
       </c>
       <c r="H27" t="n">
-        <v>5</v>
+        <v>0.7027</v>
       </c>
       <c r="I27" t="n">
-        <v>3519</v>
+        <v>6</v>
       </c>
       <c r="J27" t="n">
-        <v>416</v>
+        <v>3554</v>
       </c>
       <c r="K27" t="n">
-        <v>24449</v>
+        <v>269</v>
+      </c>
+      <c r="L27" t="n">
+        <v>10493.8</v>
       </c>
     </row>
     <row r="28">
@@ -1749,31 +1795,34 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
           <t>La cañihua parda contiene 355 kcal por 100g según la TPCA CENAN/INS. Aporta 13.8g de proteínas, 3.5g de grasas y 66.2g de carbohidratos. IG 45. RECOMENDADO para control glucémico en DM2 por su bajo índice glucémico.</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>La cañihua parda tiene 355.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Y sí, la cañihua parda es muy beneficiosa para el control de la glucosa. Tiene un Índice Glucémico (IG) de 45, que es considerado bajo. Los alimentos con IG bajo (≤55) son recomendados para personas con diabetes tipo 2 porque liberan glucosa de manera más lenta y constante en el torrente sanguíneo, evitando picos bruscos de azúcar en la sangre.
-Además, la cañihua parda es rica en proteínas (13.8g por 100g) y fibra, lo que ayuda a ralentizar la absorción de azúcares y a mantener una sensación de saciedad por más tiempo. 
-Recuerda siempre consumir porciones adecuadas y mantener una dieta equilibrada. Consulta con tu médico o nutricionista para un plan de alimentación personalizado.</t>
-        </is>
-      </c>
-      <c r="G28" t="n">
-        <v>0.8425</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>La cañihua parda contiene 355.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, la cañihua es una excelente opción para controlar la glucosa. Tiene un Índice Glucémico (IG) de 45, lo que se considera bajo, y es rica en proteínas (13.8g) y fibra, lo que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo. Esto puede contribuir a mantener niveles de glucosa más estables después de las comidas. ¡Es una buena elección para tu dieta!</t>
+        </is>
       </c>
       <c r="H28" t="n">
-        <v>5</v>
+        <v>0.6764</v>
       </c>
       <c r="I28" t="n">
-        <v>3382</v>
+        <v>6</v>
       </c>
       <c r="J28" t="n">
-        <v>255</v>
+        <v>3552</v>
       </c>
       <c r="K28" t="n">
-        <v>16169</v>
+        <v>126</v>
+      </c>
+      <c r="L28" t="n">
+        <v>9750.1</v>
       </c>
     </row>
     <row r="29">
@@ -1795,28 +1844,33 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
           <t>La kiwicha o amaranto contiene 351 kcal por 100g según la TPCA CENAN/INS 2025. Aporta 12.8g de proteínas, 6.6g de grasas y 69.1g de carbohidratos. Tiene 9.3g de fibra dietaria. IG 35, bajo.</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>La Kiwicha o Amaranto tiene 351.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.</t>
-        </is>
-      </c>
-      <c r="G29" t="n">
-        <v>0.8592</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>La kiwicha contiene 351 kcal por 100g según la TPCA CENAN/INS.</t>
+        </is>
       </c>
       <c r="H29" t="n">
+        <v>0.6744</v>
+      </c>
+      <c r="I29" t="n">
         <v>5</v>
       </c>
-      <c r="I29" t="n">
-        <v>3527</v>
-      </c>
       <c r="J29" t="n">
-        <v>58</v>
+        <v>3446</v>
       </c>
       <c r="K29" t="n">
-        <v>15720</v>
+        <v>22</v>
+      </c>
+      <c r="L29" t="n">
+        <v>6202.1</v>
       </c>
     </row>
     <row r="30">
@@ -1834,38 +1888,38 @@
         <v>351</v>
       </c>
       <c r="D30" t="n">
-        <v>410</v>
+        <v>351</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
           <t>La kiwicha tiene 351 kcal/100g con IG 35, menor que la quinua (IG 53). Ambas tienen similar contenido calórico pero la kiwicha tiene mayor fibra (9.3g vs 5.9g). RECOMENDADO para DM2. El menor IG de la kiwicha produce menor pico glucémico postprandial.</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>La kiwicha es un alimento muy nutritivo y beneficioso para las personas con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, la kiwicha tiene las siguientes características:
-- Energía: Entre 351 y 410 kcal por 100g de porción comestible, dependiendo de la forma en que se prepare (precocida, tostada, en harina, pop).
-- Índice Glucémico (IG): 35, lo que se considera bajo y es recomendado para personas con diabetes.
-Comparándola con la quinua, que tiene un IG de 53 y aporta alrededor de 368 kcal por 100g, la kiwicha tiene un IG más bajo, lo que significa que su consumo produce un aumento más lento y menor de la glucosa en sangre, lo cual es beneficioso en DM2.
-Además, la kiwicha es rica en proteínas y fibra dietaria, lo que ayuda a controlar la glucosa en sangre y aporta saciedad, ayudando en el control del peso.
-Sin embargo, tanto la kiwicha como la quinua son excelentes opciones para incluir en la dieta de una persona con diabetes tipo 2. Ambos son cereales andinos ricos en nutrientes y con un IG bajo o moderado. La elección entre uno u otro puede depender de tus preferencias de sabor, disponibilidad o costo.
-Recuerda siempre mantener una porción adecuada para no exceder la cantidad de carbohidratos recomendada por comida (máximo 45.0g). Consulta con tu médico o nutricionista para determinar la porción adecuada para ti.</t>
-        </is>
-      </c>
-      <c r="G30" t="n">
-        <v>0.832</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>La kiwicha contiene 351 kcal por 100g según la TPCA CENAN/INS, y su índice glucémico (IG) es de 35, lo que la clasifica como un alimento de IG bajo, recomendado para diabetes.
+Comparando con la quinua, que tiene un IG de 53 (medio), la kiwicha es mejor para personas con diabetes tipo 2 debido a su menor índice glucémico. Esto significa que la kiwicha puede ayudar a mantener niveles de glucosa más estables en sangre. Además, la kiwicha es rica en proteínas y fibra, lo que también contribuye a un mejor control glucémico.</t>
+        </is>
       </c>
       <c r="H30" t="n">
+        <v>0.6758999999999999</v>
+      </c>
+      <c r="I30" t="n">
         <v>5</v>
       </c>
-      <c r="I30" t="n">
-        <v>3583</v>
-      </c>
       <c r="J30" t="n">
-        <v>390</v>
+        <v>3454</v>
       </c>
       <c r="K30" t="n">
-        <v>30932</v>
+        <v>138</v>
+      </c>
+      <c r="L30" t="n">
+        <v>11994.7</v>
       </c>
     </row>
     <row r="31">
@@ -1887,33 +1941,35 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
           <t>La kiwicha pop o reventada mantiene un perfil calórico similar (~351 kcal/100g) según la TPCA. Al no agregar azúcar es RECOMENDADO como snack para DM2. Aportar fibra y proteínas que reducen el hambre entre comidas. Porción: 30g.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>La Kiwicha pop o reventada tiene aproximadamente 410 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Además, la Kiwicha pop es un excelente snack para personas con diabetes tipo 2. Tiene un Índice Glucémico (IG) de 35, lo que se considera bajo. Los alimentos con un IG bajo son más lentos para liberar glucosa en la sangre, lo que ayuda a mantener los niveles de azúcar en la sangre más estables.
-Además, la Kiwicha pop es rica en proteínas (14g por 100g) y tiene un buen contenido de fibra, lo que contribuye a una sensación de saciedad y ayuda a controlar el apetito.
-Recuerda que, aunque es un snack saludable, debes controlar las porciones para no exceder la cantidad recomendada de carbohidratos por comida (45g). Por ejemplo, si consumes 30g de Kiwicha pop, estarías consumiendo alrededor de 22g de carbohidratos.
-Siempre es importante leer las etiquetas de los productos comerciales de Kiwicha pop, ya que algunos pueden contener azúcares añadidos u otros ingredientes no recomendables para personas con diabetes. 
-Y recuerda, cada persona con diabetes es única. Lo que funciona para uno, puede no funcionar para otro. Es importante monitorear tus niveles de azúcar en la sangre y trabajar con tu equipo de atención médica para determinar qué alimentos son los mejores para ti.</t>
-        </is>
-      </c>
-      <c r="G31" t="n">
-        <v>0.8265</v>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>La kiwicha pop de Lima contiene 410.0 kcal por 100g según la TPCA CENAN/INS. 
+En cuanto a si es un buen snack para diabéticos, la kiwicha tiene un Índice Glucémico (IG) de 35, lo que la clasifica como un alimento de IG bajo, recomendado para personas con diabetes. Además, es rica en proteínas (14g) y contiene fibra, lo que ayuda a ralentizar la absorción de glucosa en el organismo. 
+Sin embargo, es importante consumirla en porciones controladas y dentro de un contexto de alimentación balanceada. Siempre es recomendable consultar con un médico o nutricionista antes de hacer cambios en la dieta.</t>
+        </is>
       </c>
       <c r="H31" t="n">
+        <v>0.6126</v>
+      </c>
+      <c r="I31" t="n">
         <v>5</v>
       </c>
-      <c r="I31" t="n">
-        <v>3547</v>
-      </c>
       <c r="J31" t="n">
-        <v>368</v>
+        <v>3449</v>
       </c>
       <c r="K31" t="n">
-        <v>14151</v>
+        <v>148</v>
+      </c>
+      <c r="L31" t="n">
+        <v>7560.7</v>
       </c>
     </row>
     <row r="32">
@@ -1931,66 +1987,65 @@
         <v>351</v>
       </c>
       <c r="D32" t="n">
-        <v>220</v>
+        <v>376</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
           <t>Desayuno RECOMENDADO para DM2: Quinua (351 kcal/100g, IG 53) con leche fresca (62 kcal/100g, IG 27). Combinar 50g de quinua cocida (89 kcal) + 200ml leche = ~200 kcal totales. Esta combinación aporta proteínas completas y calcio sin elevar la glucosa bruscamente.</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>¡Claro que sí! Aquí te dejo una receta de desayuno saludable y deliciosa con quinua para un paciente con diabetes tipo 2.
-🍽️ **Desayuno de Quinua con Frutas**
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>La quinua contiene 376 kcal por 100g según la TPCA CENAN/INS. 
+🍽️ **Desayuno de Quinua con Frutas y Yogur**
 ⏱️ Tiempo: 20 minutos | Dificultad: fácil
-💰 **Accesibilidad:** 🟡 Moderado
+💰 **Accesibilidad:** 🟢 Económico
 📋 **Ingredientes:**
-- Quinua cocida (1 taza)
-- Leche descremada (1 taza)
-- Manzana (1/2 unidad)
-- Fresas (1/2 taza)
-- Canela (al gusto)
+- 50g de quinua cocida
+- 100g de yogur natural sin azúcar
+- 50g de aguaymanto (o cualquier fruta de bajo IG como fresas o arándanos)
 👨‍🍳 **Preparación:**
-1. Cocina la quinua en agua hasta que esté suave y esponjosa. Escurre el exceso de agua.
-2. En una olla, añade la leche descremada y la quinua cocida. Cocina a fuego medio hasta que la mezcla esté caliente.
-3. Agrega la manzana picada y las fresas. Cocina por unos minutos más hasta que las frutas estén suaves.
-4. Sirve caliente y espolvorea con un poco de canela.
+1. Cocina la quinua en agua (1 parte de quinua por 2 partes de agua) durante 15 minutos hasta que esté suave. Escurre y deja enfriar.
+2. En un tazón, mezcla la quinua cocida con el yogur natural.
+3. Agrega el aguaymanto (o la fruta elegida) encima y mezcla suavemente.
 🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: Manzana y fresas
-2.° Luego: Quinua con leche
-3.° Al final: No aplica en este caso
+1.° Come primero: **aguaymanto** (o la fruta elegida)
+2.° Luego: **yogur con quinua**
+3.° Al final: **más aguaymanto si deseas**
 📊 **Información nutricional estimada (por porción):**
 - Calorías: 220 kcal
-- Carbohidratos: 40g
-- Proteínas: 8g
-- Grasas: 3g
+- Carbohidratos: 30g
+- Proteínas: 10g
+- Grasas: 4g
 - Fibra: 5g
-- IG estimado: 53 (bajo)
+- IG estimado: Bajo
 🧠 **¿Por qué esta receta es buena para ti?**
-La quinua es un grano andino con un Índice Glucémico bajo (IG=53), lo que significa que su azúcar se libera lentamente en el torrente sanguíneo, evitando picos de glucosa. Además, es rica en proteínas y fibra, que ayudan a mantener la saciedad. Las manzanas y las fresas añaden fibra adicional y antioxidantes beneficiosos.
+La quinua (IG=53) aporta proteínas y fibra, lo que ayuda a regular la glucosa en sangre. El yogur natural sin azúcar proporciona probióticos que benefician la salud digestiva, y el aguaymanto es rico en antioxidantes y tiene un IG bajo, lo que lo hace ideal para tu desayuno.
 💡 **Tips DM2:**
-- Recuerda que la porción recomendada de frutas para un paciente con DM2 es de 1 a 2 porciones al día.
-- Puedes variar las frutas según la temporada y tu preferencia, siempre y cuando sean bajas en azúcar.
+- Puedes variar las frutas según la temporada y disponibilidad, siempre eligiendo aquellas con bajo IG.
 🔄 **Alternativas:**
-- Si no tienes manzana, puedes usar pera o durazno.
-- Si no tienes fresas, puedes usar arándanos o frambuesas.
-Según los datos de la TPCA del CENAN/INS, la quinua cocida tiene aproximadamente 89.0 kcal por cada 100g.</t>
-        </is>
-      </c>
-      <c r="G32" t="n">
-        <v>0.8263</v>
+- Si no tienes aguaymanto, puedes usar fresas o arándanos, que también son opciones de bajo IG.</t>
+        </is>
       </c>
       <c r="H32" t="n">
-        <v>5</v>
+        <v>0.6254999999999999</v>
       </c>
       <c r="I32" t="n">
-        <v>3442</v>
+        <v>7</v>
       </c>
       <c r="J32" t="n">
-        <v>660</v>
+        <v>3842</v>
       </c>
       <c r="K32" t="n">
-        <v>37644</v>
+        <v>475</v>
+      </c>
+      <c r="L32" t="n">
+        <v>11118.3</v>
       </c>
     </row>
     <row r="33">
@@ -2012,60 +2067,61 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
           <t>Desayuno RECOMENDADO para DM2: Avena hojuela (333 kcal/100g, IG 55) + aguaymanto (53 kcal, IG 25). Preparar 40g de avena cocida (~130 kcal) + 100g aguaymanto (53 kcal) = ~183 kcal totales. El beta-glucano de la avena ralentiza la absorción de glucosa; el aguaymanto aporta vitamina C y antioxidantes.</t>
         </is>
       </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>La avena es un alimento muy recomendado para personas con diabetes tipo 2 debido a su bajo Índice Glucémico (IG=55) y su alto contenido de fibra, que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, la avena cocida proporciona aproximadamente 54.0 kcal por cada 100g, mientras que la avena envasada proporciona alrededor de 380.0 kcal por cada 100g.
-Aquí te dejo una receta de desayuno con avena especialmente diseñada para personas con diabetes tipo 2:
-🍽️ **Desayuno de Avena con Frutas**
-⏱️ Tiempo: 15 minutos | Dificultad: fácil
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>La avena contiene 54.0 kcal por 100g según la TPCA CENAN/INS.
+🍽️ **Desayuno de Avena con Frutas y Semillas**
+⏱️ Tiempo: 10 minutos | Dificultad: fácil
 💰 **Accesibilidad:** 🟢 Económico
 📋 **Ingredientes:**
-- Avena cocida (1 taza)
-- Manzana (1/2 unidad)
-- Fresas (1/2 taza)
-- Almendras (10 unidades)
+- 50g de avena (hojuela cocida)
+- 1/2 plátano (50g)
+- 1 cucharada de semillas de chía (15g)
+- 1 taza de agua o leche descremada (250ml)
 👨‍🍳 **Preparación:**
-1. Cocina la avena en agua hasta que esté suave.
-2. Corta la manzana y las fresas en trozos pequeños.
-3. Mezcla la avena cocida con las frutas y las almendras.
+1. Cocina la avena en agua o leche a fuego medio durante 5-7 minutos hasta que esté suave.
+2. Sirve en un tazón y agrega el plátano cortado en rodajas y las semillas de chía por encima.
 🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: Manzana y fresas
-2.° Luego: Almendras
-3.° Al final: Avena
+1.° Come primero: **ensalada de frutas** (puedes agregar otras frutas bajas en azúcar como fresas o aguaymanto).
+2.° Luego: **avena**.
+3.° Al final: **semillas de chía**.
 📊 **Información nutricional estimada (por porción):**
-- Calorías: Aproximadamente 250 kcal
-- Carbohidratos: 30g
+- Calorías: 210 kcal
+- Carbohidratos: 35g
 - Proteínas: 7g
-- Grasas: 10g
-- Fibra: 7g
+- Grasas: 4g
+- Fibra: 8g
 - IG estimado: Bajo
 🧠 **¿Por qué esta receta es buena para ti?**
-La avena tiene un bajo IG y es rica en fibra, lo que ayuda a controlar los niveles de glucosa en la sangre. Las manzanas y las fresas son frutas de bajo IG que aportan vitaminas y antioxidantes. Las almendras aportan proteínas y grasas saludables que también ayudan a regular la glucemia.
+La avena (IG=55) es rica en fibra soluble, lo que ayuda a regular los niveles de glucosa en sangre. Las semillas de chía aportan ácidos grasos omega-3 y más fibra, lo que también contribuye a una mejor salud digestiva y control glucémico.
 💡 **Tips DM2:**
-- Recuerda que el tamaño de las porciones es importante. Asegúrate de no exceder la cantidad recomendada de carbohidratos por comida (45g).
-- Si prefieres la avena envasada, recuerda que tiene más calorías que la avena cocida, así que ajusta la porción en consecuencia.
+- Puedes variar las frutas según la temporada y tus preferencias, pero siempre elige opciones con bajo índice glucémico.
 🔄 **Alternativas:**
-- Si no tienes fresas, puedes usar otras frutas de bajo IG como peras o duraznos.
-- Si no tienes almendras, puedes usar nueces o semillas de chía.</t>
-        </is>
-      </c>
-      <c r="G33" t="n">
-        <v>0.8256</v>
+- Si no tienes plátano, puedes usar manzana o pera, que también son buenas opciones.</t>
+        </is>
       </c>
       <c r="H33" t="n">
-        <v>5</v>
+        <v>0.5633</v>
       </c>
       <c r="I33" t="n">
-        <v>3537</v>
+        <v>6</v>
       </c>
       <c r="J33" t="n">
-        <v>685</v>
+        <v>3688</v>
       </c>
       <c r="K33" t="n">
-        <v>26992</v>
+        <v>459</v>
+      </c>
+      <c r="L33" t="n">
+        <v>11638.3</v>
       </c>
     </row>
     <row r="34">
@@ -2083,69 +2139,71 @@
         <v>284</v>
       </c>
       <c r="D34" t="n">
-        <v>328</v>
+        <v>59</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
           <t>Almuerzo RECOMENDADO para DM2: Cebada perlada (284 kcal cruda, IG 28) + brócoli (34 kcal) + zanahoria (44 kcal). 50g cebada cocida (~30 kcal) + 100g brócoli + 50g zanahoria = ~100 kcal del plato base. La cebada con fibra 17.3g es el cereal más favorable para DM2 por su IG 28 ultra bajo.</t>
         </is>
       </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>La cebada es un alimento muy recomendado para personas con diabetes tipo 2 debido a su bajo Índice Glucémico (IG=28) y su alto contenido de fibra dietaria, lo que ayuda a ralentizar la absorción de glucosa en el organismo. 
-Aquí te dejo una receta saludable y económica con cebada:
-🍽️ **Ensalada de cebada con verduras**
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>La cebada es una excelente opción para un almuerzo saludable en personas con diabetes. La cebada perlada o resbalada cocida contiene 59.0 kcal por 100g según la TPCA CENAN/INS.
+🍽️ **Ensalada de Cebada con Verduras**
 ⏱️ Tiempo: 30 minutos | Dificultad: fácil
 💰 **Accesibilidad:** 🟢 Económico
 📋 **Ingredientes:**
-- Cebada pelada (1 taza)
-- Zanahoria (1 unidad)
-- Pimiento rojo (1/2 unidad)
-- Espinaca (1 taza)
-- Aceite de oliva (1 cucharada)
-- Jugo de limón (al gusto)
-- Sal (al gusto)
+- 100g de cebada perlada cocida
+- 1 taza de espinacas frescas
+- 1/2 taza de tomate en cubos
+- 1/4 de cebolla morada en rodajas
+- Jugo de 1 limón
+- 1 cucharada de aceite de oliva
+- Sal y pimienta al gusto
 👨‍🍳 **Preparación:**
-1. Cocina la cebada en abundante agua hasta que esté suave (aproximadamente 20 minutos). Luego, escúrrela y déjala enfriar.
-2. Pica la zanahoria y el pimiento en cubos pequeños.
-3. En un bol grande, mezcla la cebada, la zanahoria, el pimiento y la espinaca.
-4. Adereza con aceite de oliva, jugo de limón y sal al gusto. Mezcla bien y sirve.
+1. Cocina la cebada en agua hirviendo durante aproximadamente 30 minutos hasta que esté tierna. Escurre y deja enfriar.
+2. En un tazón grande, mezcla las espinacas, el tomate y la cebolla.
+3. Agrega la cebada cocida y mezcla bien.
+4. Aliña con el jugo de limón, aceite de oliva, sal y pimienta al gusto.
 🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: Espinaca
-2.° Luego: Cebada
-3.° Al final: Zanahoria y pimiento
+1.° Come primero: **Ensalada de espinacas, tomate y cebolla**
+2.° Luego: **Cebada**
+3.° Al final: **Si deseas, puedes agregar una proteína como pollo a la plancha o atún**
 📊 **Información nutricional estimada (por porción):**
-- Calorías: 328 kcal (de la cebada)
-- Carbohidratos: 73.3g
-- Proteínas: 8.2g
-- Grasas: 1.1g
-- Fibra: 17.3g (estimada)
+- Calorías: 200 kcal
+- Carbohidratos: 30g
+- Proteínas: 6g
+- Grasas: 7g
+- Fibra: 5g
 - IG estimado: 28 (bajo)
 🧠 **¿Por qué esta receta es buena para ti?**
-La cebada es una excelente fuente de fibra dietaria que ayuda a controlar los niveles de azúcar en la sangre. Además, las verduras aportan vitaminas y minerales esenciales para tu salud.
+La cebada (IG=28) es rica en fibra (3.8g por 100g), lo que ayuda a ralentizar la absorción de glucosa en el torrente sanguíneo, manteniendo niveles de azúcar más estables.
 💡 **Tips DM2:**
-- Recuerda beber suficiente agua durante el día para ayudar a la fibra a hacer su trabajo.
-- Puedes añadir un poco de proteína a esta ensalada con un huevo duro o un poco de pechuga de pollo a la plancha.
+- Puedes variar las verduras según la temporada y tus preferencias.
 🔄 **Alternativas:**
-- Si no tienes espinaca, puedes usar lechuga o acelga.
-- Si no tienes pimiento rojo, puedes usar pimiento verde o amarillo.
-Recuerda que los valores nutricionales son aproximados y pueden variar según las porciones y la forma de cocción. Consulta con tu médico o nutricionista para ajustar la receta a tus necesidades específicas.</t>
-        </is>
-      </c>
-      <c r="G34" t="n">
-        <v>0.8297</v>
+- Si no tienes espinacas, puedes usar lechuga o rúcula. 
+¡Espero que disfrutes de esta deliciosa y saludable ensalada! 🍽️</t>
+        </is>
       </c>
       <c r="H34" t="n">
-        <v>5</v>
+        <v>0.5904</v>
       </c>
       <c r="I34" t="n">
-        <v>3462</v>
+        <v>7</v>
       </c>
       <c r="J34" t="n">
-        <v>714</v>
+        <v>3838</v>
       </c>
       <c r="K34" t="n">
-        <v>16182</v>
+        <v>529</v>
+      </c>
+      <c r="L34" t="n">
+        <v>12090.6</v>
       </c>
     </row>
     <row r="35">
@@ -2163,65 +2221,67 @@
         <v>115</v>
       </c>
       <c r="D35" t="n">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
           <t>Almuerzo RECOMENDADO para DM2: Tarwi cocido (115 kcal/100g, IG 16) + ensalada de tomate (20 kcal) + palta (177 kcal). 100g tarwi + 100g tomate + 50g palta = ~225 kcal totales. El tarwi aporta 15.6g proteínas; la palta grasas monoinsaturadas que mejoran sensibilidad a insulina.</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>¡Claro que sí! Te presento una receta saludable y deliciosa de "Ensalada de Tarwi".
-🍽️ **Ensalada de Tarwi**
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>🍽️ **Ensalada de Tarwi con Verduras**
 ⏱️ Tiempo: 30 minutos | Dificultad: fácil
-💰 **Accesibilidad:** 🟢 Económico 
+💰 **Accesibilidad:** 🟢 Económico
 📋 **Ingredientes:**
-- Tarwi (lupinus mutabilis) remojado y cocido (1 taza)
-- Tomate (1 unidad)
-- Pepino (1/2 unidad)
-- Lechuga (1 taza)
+- Tarwi cocido (100g)
+- Espinaca fresca (50g)
+- Tomate (50g)
+- Cebolla roja (30g)
+- Limón (al gusto)
 - Aceite de oliva (1 cucharada)
-- Limón (1/2 unidad)
-- Sal al gusto
 👨‍🍳 **Preparación:**
-1. Lava y corta el tomate, el pepino y la lechuga en trozos pequeños.
-2. En un bol, mezcla el tarwi cocido con los vegetales cortados.
-3. Adereza con el aceite de oliva, el jugo de limón y la sal al gusto. 
+1. Cocina el tarwi en agua hirviendo durante aproximadamente 30 minutos hasta que esté tierno. Escurre y deja enfriar.
+2. Lava bien las espinacas, el tomate y la cebolla. Corta el tomate y la cebolla en rodajas finas.
+3. En un bol, mezcla el tarwi cocido, las espinacas, el tomate y la cebolla.
+4. Aliña con jugo de limón y aceite de oliva al gusto.
 🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: Lechuga, tomate y pepino
-2.° Luego: Tarwi
-3.° Al final: No hay carbohidratos en esta receta
+1.° Come primero: **Espinacas, tomate y cebolla** (ensalada)
+2.° Luego: **Tarwi** (proteína)
+3.° Al final: **Ningún carbohidrato adicional** en esta receta.
 📊 **Información nutricional estimada (por porción):**
-- Calorías: 250 kcal
-- Carbohidratos: 15g
-- Proteínas: 20g
+- Calorías: 210 kcal
+- Carbohidratos: 20g
+- Proteínas: 12g
 - Grasas: 10g
-- Fibra: 5g
+- Fibra: 7g
 - IG estimado: 15 (bajo)
-🧠 **¿Por qué esta receta es buena para ti?**
-El tarwi es una legumbre peruana con un índice glucémico muy bajo (IG=15), lo que significa que su consumo no eleva rápidamente los niveles de azúcar en la sangre. Además, es rico en proteínas y fibra, lo que ayuda a controlar la glucemia y a mantener la sensación de saciedad.
-💡 **Tips DM2:**
-- Recuerda remojar el tarwi durante al menos una noche para eliminar los alcaloides amargos antes de cocinarlo.
-- Puedes añadir otras verduras de tu preferencia para variar la ensalada.
+💡 **¿Por qué esta receta es buena para ti?**
+El tarwi (IG=15) es excelente para personas con diabetes, ya que es rico en proteínas (12g) y fibra (7g), lo que ayuda a controlar los niveles de glucosa en sangre al ralentizar la absorción de azúcares. Además, las espinacas y el tomate aportan antioxidantes y vitaminas esenciales.
 🔄 **Alternativas:**
-- Si no tienes tarwi, puedes usar lentejas o garbanzos, pero ten en cuenta que estos tienen un índice glucémico más alto.</t>
-        </is>
-      </c>
-      <c r="G35" t="n">
-        <v>0.8139</v>
+- Si no tienes tarwi, puedes usar **lentejas** o **guisantes** como fuente de proteína.
+¡Espero que disfrutes de esta deliciosa y saludable ensalada! ¡Cada comida bien elegida cuenta! 😊</t>
+        </is>
       </c>
       <c r="H35" t="n">
-        <v>5</v>
+        <v>0.5567</v>
       </c>
       <c r="I35" t="n">
-        <v>3392</v>
+        <v>10</v>
       </c>
       <c r="J35" t="n">
-        <v>564</v>
+        <v>4294</v>
       </c>
       <c r="K35" t="n">
-        <v>22960</v>
+        <v>482</v>
+      </c>
+      <c r="L35" t="n">
+        <v>12012.6</v>
       </c>
     </row>
     <row r="36">
@@ -2239,61 +2299,63 @@
         <v>53</v>
       </c>
       <c r="D36" t="n">
-        <v>155</v>
+        <v>51</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
           <t>Merienda RECOMENDADO para DM2: Aguaymanto fresco (53 kcal/100g, IG 25) + cañihua pop (381 kcal cruda). 100g aguaymanto + 20g cañihua pop = ~130 kcal. Esta combinación andina aporta vitamina C, hierro y proteínas vegetales con bajo impacto glucémico.</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr">
-        <is>
-          <t>¡Claro! Aquí te dejo una receta de merienda saludable con aguaymanto, ideal para personas con diabetes tipo 2.
-🍽️ **Ensalada de Aguaymanto y Avena**
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>🍽️ **Merienda de Aguaymanto con Yogur Natural**
 ⏱️ Tiempo: 10 minutos | Dificultad: fácil
 💰 **Accesibilidad:** 🟢 Económico
 📋 **Ingredientes:**
-- 1 taza de aguaymanto (100g)
-- 1/2 taza de avena cocida (50g)
-- 1 cucharada de miel de abeja pura (opcional)
+- 100g de aguaymanto
+- 150g de yogur natural sin azúcar
 👨‍🍳 **Preparación:**
-1. Cocina la avena en agua hasta que esté suave.
-2. Lava bien los aguaymantos y córtalos por la mitad.
-3. Mezcla la avena cocida con los aguaymantos en un tazón.
-4. Si lo deseas, puedes endulzar ligeramente con una cucharada de miel de abeja pura.
+1. Lava bien los aguaymantos y colócalos en un tazón.
+2. Agrega el yogur natural por encima de los aguaymantos.
+3. Mezcla suavemente y disfruta.
 🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: Aguaymanto
-2.° Luego: Avena
+1.° Come primero: aguaymanto
+2.° Luego: yogur natural
 📊 **Información nutricional estimada (por porción):**
-- Calorías: 155 kcal
-- Carbohidratos: 33.7g
-- Proteínas: 3.2g
-- Grasas: 1.8g
+- Calorías: 116 kcal (51 kcal del aguaymanto + 65 kcal del yogur)
+- Carbohidratos: 15.3g
+- Proteínas: 6.3g
+- Grasas: 2.5g
 - Fibra: 4.9g
-- IG estimado: 40 (bajo)
+- IG estimado: 25 (bajo)
 🧠 **¿Por qué esta receta es buena para ti?**
-El aguaymanto tiene un Índice Glucémico (IG) de 25, lo que significa que su azúcar se libera lentamente en la sangre, evitando picos de glucosa. Además, es rico en vitamina C y fibra. La avena, por otro lado, tiene un IG de 55 y es una excelente fuente de fibra que ayuda a controlar los niveles de azúcar en la sangre.
+El aguaymanto (IG=25) es una fruta con bajo índice glucémico, rica en fibra (4.9g), lo que ayuda a controlar los niveles de azúcar en sangre. Además, el yogur natural aporta proteínas y probióticos que favorecen la salud intestinal.
 💡 **Tips DM2:**
-- Recuerda que la miel de abeja, aunque natural, es un azúcar simple. Si decides usarla, hazlo con moderación y siempre ten en cuenta la cantidad total de carbohidratos que estás consumiendo.
+- Opta por yogur natural sin azúcar para evitar picos de glucosa.
 🔄 **Alternativas:**
-- Si no tienes aguaymanto, puedes usar frutas con IG bajo como las fresas o manzanas. 
-Recuerda siempre consultar a tu médico o nutricionista antes de hacer cambios en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G36" t="n">
-        <v>0.8162</v>
+- Si no tienes aguaymanto, puedes usar fresas o arándanos, que también son frutas con bajo IG.
+Además, el aguaymanto contiene 51.0 kcal por 100g según la TPCA CENAN/INS. ¡Disfruta de esta merienda saludable!</t>
+        </is>
       </c>
       <c r="H36" t="n">
-        <v>5</v>
+        <v>0.5993000000000001</v>
       </c>
       <c r="I36" t="n">
-        <v>3463</v>
+        <v>6</v>
       </c>
       <c r="J36" t="n">
-        <v>599</v>
+        <v>3648</v>
       </c>
       <c r="K36" t="n">
-        <v>24157</v>
+        <v>422</v>
+      </c>
+      <c r="L36" t="n">
+        <v>10601.8</v>
       </c>
     </row>
     <row r="37">
@@ -2311,135 +2373,116 @@
         <v>124</v>
       </c>
       <c r="D37" t="n">
-        <v>159</v>
+        <v>127</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
           <t>Cena RECOMENDADA para DM2: Jurel fresco (124 kcal/100g, IG 0) + brócoli al vapor (34 kcal). 150g jurel + 150g brócoli = ~230 kcal totales. El omega-3 del jurel mejora sensibilidad a insulina; el brócoli aporta fibra y vitamina C sin elevar glucosa.</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>El jurel a la plancha es una excelente opción para la cena de un paciente con diabetes tipo 2. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, 100g de jurel a la plancha (o frito en aceite vegetal sin sal) tiene aproximadamente 159 kcal. Además, tiene un Índice Glucémico (IG) de 0, lo que significa que no aumenta rápidamente los niveles de azúcar en la sangre.
-🍽️ **Jurel a la Plancha**
-⏱️ Tiempo: 15 minutos | Dificultad: fácil
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>No tengo el dato exacto en la TPCA sobre el jurel a la plancha. Sin embargo, puedo decirte que el pescado jurel fresco contiene 121.0 kcal por 100g según la TPCA CENAN/INS.
+El jurel es una excelente opción para la cena en personas con diabetes. Tiene un Índice Glucémico (IG) de 0, lo que significa que no eleva los niveles de glucosa en sangre. Además, es rico en proteínas (22.2g por 100g) y bajo en grasas (2.7g por 100g), lo que ayuda a mantener la saciedad y a controlar el peso.
+Te recomiendo acompañarlo con una buena porción de verduras al vapor o una ensalada fresca para maximizar los beneficios y seguir el orden de consumo adecuado. ¡Es una opción deliciosa y saludable! 🍽️</t>
+        </is>
+      </c>
+      <c r="H37" t="n">
+        <v>0.4872</v>
+      </c>
+      <c r="I37" t="n">
+        <v>7</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3432</v>
+      </c>
+      <c r="K37" t="n">
+        <v>182</v>
+      </c>
+      <c r="L37" t="n">
+        <v>11313.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Colación palta + tomate</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>¿Qué colación con palta es recomendada para un paciente con diabetes tipo 2? ¿Cuántas calorías tiene la palta?</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>177</v>
+      </c>
+      <c r="D38" t="n">
+        <v>166</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Colación RECOMENDADA para DM2: Palta (177 kcal/100g, IG 15) con tomate cherry (20 kcal). 50g palta (~90 kcal) + 100g tomate (20 kcal) = ~110 kcal. La palta aporta grasas monoinsaturadas que mejoran perfil lipídico; el tomate licopenos antioxidantes.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>La palta contiene 130 kcal por 100g según la TPCA CENAN/INS. 
+🍽️ **Colación de Palta con Limón y Sal**
+⏱️ Tiempo: 5 minutos | Dificultad: fácil
 💰 **Accesibilidad:** 🟢 Económico
 📋 **Ingredientes:**
-- Jurel (200g)
-- Aceite de oliva (1 cucharada)
-- Sal y pimienta al gusto
-- Limón (opcional)
+- 100g de palta (1/2 palta mediana)
+- Jugo de 1/2 limón
+- Sal al gusto (opcional)
 👨‍🍳 **Preparación:**
-1. Calienta la plancha y añade una cucharada de aceite de oliva.
-2. Sazona el jurel con sal y pimienta al gusto.
-3. Cocina el jurel en la plancha durante unos 7 minutos por cada lado.
-4. Sirve caliente y puedes añadir unas gotas de limón si lo deseas.
+1. Corta la palta por la mitad, quita el hueso y saca la pulpa con una cuchara.
+2. Coloca la pulpa en un plato y aplástala ligeramente con un tenedor.
+3. Agrega el jugo de limón y mezcla bien. Si deseas, añade un poco de sal al gusto.
 🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: una ensalada verde
-2.° Luego: el jurel a la plancha
-3.° Al final: si deseas añadir un carbohidrato, opta por una pequeña porción de quinua o camote.
+1.° Come primero: [puedes acompañar con rodajas de pepino o zanahoria como vegetales]
+2.° Luego: [la palta]
+3.° Al final: [puedes incluir galletas integrales o un puñado de nueces]
 📊 **Información nutricional estimada (por porción):**
-- Calorías: 318 kcal
-- Carbohidratos: 0g
-- Proteínas: 53.6g
-- Grasas: 7.8g
-- Fibra: 0g
-- IG estimado: 0 (bajo)
-🧠 **¿Por qué esta receta es buena para ti?**
-El jurel es una excelente fuente de proteína y tiene un IG de 0, lo que significa que no aumentará rápidamente tus niveles de azúcar en la sangre. Además, es rico en omega-3, beneficioso para la salud del corazón.
-💡 **Tips DM2:**
-- Recuerda que la cena debe ser más ligera que el almuerzo. Si añades un carbohidrato, asegúrate de que sea una porción pequeña.
-- Siempre es buena idea acompañar tus comidas con una ensalada verde.
-🔄 **Alternativas:**
-- Si no tienes jurel, puedes usar otro pescado de tu preferencia, siempre y cuando sea bajo en grasa.</t>
-        </is>
-      </c>
-      <c r="G37" t="n">
-        <v>0.8118</v>
-      </c>
-      <c r="H37" t="n">
-        <v>5</v>
-      </c>
-      <c r="I37" t="n">
-        <v>3365</v>
-      </c>
-      <c r="J37" t="n">
-        <v>638</v>
-      </c>
-      <c r="K37" t="n">
-        <v>23838</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="inlineStr">
-        <is>
-          <t>Colación palta + tomate</t>
-        </is>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>¿Qué colación con palta es recomendada para un paciente con diabetes tipo 2? ¿Cuántas calorías tiene la palta?</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>177</v>
-      </c>
-      <c r="D38" t="n">
-        <v>230</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Colación RECOMENDADA para DM2: Palta (177 kcal/100g, IG 15) con tomate cherry (20 kcal). 50g palta (~90 kcal) + 100g tomate (20 kcal) = ~110 kcal. La palta aporta grasas monoinsaturadas que mejoran perfil lipídico; el tomate licopenos antioxidantes.</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>🍽️ **Tostada de Palta con Huevo Cocido**
-⏱️ Tiempo: 15 minutos | Dificultad: fácil
-💰 **Accesibilidad:** 🟢 Económico
-📋 **Ingredientes:**
-- 1 rebanada de pan integral (30g)
-- 1/4 de palta (aprox. 50g)
-- 1 huevo
-👨‍🍳 **Preparación:**
-1. Cocina el huevo en agua hirviendo por 10 minutos para que quede duro.
-2. Mientras se cocina el huevo, tuesta la rebanada de pan integral.
-3. Corta la palta en rodajas finas o aplástala con un tenedor.
-4. Una vez que el huevo esté cocido, pélalo y córtalo en rodajas.
-5. Unta la palta sobre la tostada y coloca encima las rodajas de huevo.
-🥦 **Orden de consumo (Food Sequencing):**
-1.° Come primero: [palta]
-2.° Luego: [huevo]
-3.° Al final: [pan integral]
-📊 **Información nutricional estimada (por porción):**
-- Calorías: 230 kcal (130 kcal de la palta y 100 kcal del huevo)
-- Carbohidratos: 15g (5.6g de la palta y 1g del pan integral)
-- Proteínas: 7g (1.7g de la palta y 6g del huevo)
-- Grasas: 17g (12.5g de la palta y 5g del huevo)
-- Fibra: 3g (2g de la palta y 1g del pan integral)
+- Calorías: 130 kcal
+- Carbohidratos: 5.6g
+- Proteínas: 1.7g
+- Grasas: 12.5g
+- Fibra: 6.6g
 - IG estimado: 15 (bajo)
 🧠 **¿Por qué esta receta es buena para ti?**
-La palta es una excelente opción para los pacientes con diabetes tipo 2 debido a su bajo índice glucémico (IG=15), lo cual significa que su consumo no provoca un aumento brusco de los niveles de azúcar en la sangre. Además, es rica en grasas saludables que ayudan a mantener la sensación de saciedad. El huevo aporta proteínas de alta calidad, y el pan integral añade fibra que ayuda a controlar la glucemia.
+La palta es rica en grasas saludables (ácidos grasos monoinsaturados) que ayudan a mejorar el perfil lipídico y a mantener la saciedad. Además, su bajo índice glucémico (IG=15) significa que no elevará rápidamente tus niveles de glucosa en sangre.
 💡 **Tips DM2:**
-- Recuerda que el tamaño de la porción es importante, así que limita la cantidad de palta a 1/4 por colación para mantener un balance calórico.
+- Puedes variar el acompañamiento de la palta con otros vegetales frescos para aumentar la fibra y los nutrientes.
 🔄 **Alternativas:**
-- Si no tienes pan integral, puedes usar pan de centeno o de avena. Si no tienes huevo, puedes usar atún en agua o pechuga de pollo cocida.</t>
-        </is>
-      </c>
-      <c r="G38" t="n">
-        <v>0.8176</v>
+- Si no tienes limón, puedes usar vinagre balsámico o simplemente disfrutarla sola. 
+¡Espero que disfrutes de esta colación saludable! 🍏</t>
+        </is>
       </c>
       <c r="H38" t="n">
-        <v>5</v>
+        <v>0.5407999999999999</v>
       </c>
       <c r="I38" t="n">
-        <v>3609</v>
+        <v>7</v>
       </c>
       <c r="J38" t="n">
-        <v>631</v>
+        <v>4011</v>
       </c>
       <c r="K38" t="n">
-        <v>17014</v>
+        <v>482</v>
+      </c>
+      <c r="L38" t="n">
+        <v>12018.9</v>
       </c>
     </row>
     <row r="39">
@@ -2461,31 +2504,34 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
           <t>Bebida RECOMENDADA para DM2: Camu camu (17 kcal/100g, IG muy bajo) + maracuyá (67 kcal, IG 30). Esta combinación aporta vitamina C excepcional (&gt;2000mg desde el camu camu) y fibra del maracuyá. Sin azúcar agregada. Total: ~30 kcal por vaso. Ideal para control glucémico.</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>El camu-camu es una fruta peruana que por cada 100g de porción comestible aporta 24.0 kcal. Esta fruta es altamente recomendada para pacientes con diabetes tipo 2 debido a su bajo contenido de carbohidratos (5.9g) y su alto contenido de vitamina C (2780.0mg), lo que la convierte en un excelente antioxidante.
-Si decides preparar una bebida con camu-camu, recuerda no agregar azúcar. Puedes endulzarla con un edulcorante natural como la stevia si lo prefieres. 
-Además, si sigues la secuenciación alimentaria, puedes consumir esta bebida después de tus proteínas y vegetales para mantener un mejor control de tu glucemia. 
-Recuerda siempre consultar con tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G39" t="n">
-        <v>0.8249</v>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>El camu camu contiene 24.0 kcal por 100g según la TPCA CENAN/INS. 
+En cuanto a su consumo, el camu camu es una fruta recomendada para personas con diabetes mellitus tipo 2, ya que tiene un bajo contenido calórico y es rico en vitamina C. Sin embargo, si se refiere a un refresco de camu camu con azúcar, este no sería recomendable debido a la presencia de azúcares añadidos. Siempre es mejor optar por el camu camu fresco o en preparaciones sin azúcares añadidos. ¡Consulta con tu médico antes de hacer cambios en tu dieta!</t>
+        </is>
       </c>
       <c r="H39" t="n">
-        <v>5</v>
+        <v>0.5198</v>
       </c>
       <c r="I39" t="n">
-        <v>3378</v>
+        <v>6</v>
       </c>
       <c r="J39" t="n">
-        <v>200</v>
+        <v>3259</v>
       </c>
       <c r="K39" t="n">
-        <v>8149</v>
+        <v>136</v>
+      </c>
+      <c r="L39" t="n">
+        <v>7861.4</v>
       </c>
     </row>
     <row r="40">
@@ -2507,31 +2553,34 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>La lúcuma fresca contiene 99 kcal por 100g según la TPCA. IG 25, bajo. RECOMENDADO como postre natural para DM2 en porciones de 100g. Aporta 2.3g de fibra y niacina. Sustituto natural del azúcar en preparaciones.</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>La lúcuma fresca tiene 97.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS. Además, posee un Índice Glucémico (IG) de 40, lo que es considerado bajo. Esto significa que su consumo no eleva rápidamente los niveles de glucosa en sangre, lo cual es beneficioso para personas con diabetes.
-Por lo tanto, la lúcuma puede ser un buen ingrediente para postres para personas con diabetes, siempre y cuando se consuma con moderación y se tenga en cuenta el total de carbohidratos de la comida. Recuerda que para este paciente, el límite es de 45.0g de carbohidratos por comida.
-Además, la lúcuma aporta fibra dietaria (10.2g por 100g), lo que ayuda a ralentizar la absorción de azúcar y a mantener una sensación de saciedad por más tiempo.
-Un postre saludable podría ser una mousse de lúcuma con leche descremada y un endulzante sin calorías, o simplemente la fruta fresca como tal. Recuerda siempre consultar con tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G40" t="n">
-        <v>0.8383</v>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>La lúcuma fresca contiene 97 kcal por 100g según la TPCA CENAN/INS. 
+Sí, la lúcuma fresca puede ser un excelente postre para diabéticos, ya que tiene un índice glucémico muy bajo (IG 25), lo que significa que no provoca picos significativos en los niveles de glucosa en sangre. Además, es rica en nutrientes y fibra, lo que la hace una opción saludable. ¡Disfrútala! 🍽️</t>
+        </is>
       </c>
       <c r="H40" t="n">
-        <v>5</v>
+        <v>0.6019</v>
       </c>
       <c r="I40" t="n">
-        <v>3461</v>
+        <v>6</v>
       </c>
       <c r="J40" t="n">
-        <v>304</v>
+        <v>3300</v>
       </c>
       <c r="K40" t="n">
-        <v>15562</v>
+        <v>99</v>
+      </c>
+      <c r="L40" t="n">
+        <v>7069.5</v>
       </c>
     </row>
     <row r="41">
@@ -2549,38 +2598,39 @@
         <v>399</v>
       </c>
       <c r="D41" t="n">
-        <v>317</v>
+        <v>351</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
           <t>Superalimentos andinos para DM2 según la TPCA: Tarwi (399 kcal, IG 16) es el mejor para DM2 por su mínimo impacto glucémico y 47g proteínas. Quinua (351 kcal, IG 53) y kiwicha (351 kcal, IG 35) son también RECOMENDADOS. La cañihua (381 kcal, IG 45) es la menos conocida pero muy nutritiva.</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>Los superalimentos andinos son una excelente opción para las personas con DM2 debido a su bajo índice glucémico y alto contenido de fibra y proteínas. Aquí te dejo la información nutricional de los que mencionaste:
-1. **Quinua, variedad Cuchiwilla (Puno)**: 317.0 kcal por 100g de porción comestible. Tiene un IG de 53, lo que es bajo y recomendado para diabetes. Además, aporta 15.2g de proteínas y 12.2g de fibra dietaria.
-2. **Kiwicha, precocida, hojuela de**: 400.0 kcal por 100g de porción comestible. Su IG es de 35, también bajo y recomendado para diabetes. Aporta 13.4g de proteínas.
-No tengo los datos del tarwi en este momento, pero es conocido por tener un IG muy bajo (15) y alto contenido de proteína vegetal.
-Para DM2, todos estos superalimentos son recomendables, pero si tuviera que elegir uno, te recomendaría la **quinua**. No solo tiene un IG bajo, sino que también aporta una buena cantidad de proteínas y fibra dietaria. La fibra ayuda a ralentizar la absorción de glucosa, lo que puede ayudar a controlar los niveles de azúcar en sangre. Además, la quinua es versátil y puede ser usada en una variedad de platos, desde desayunos hasta cenas.
-Recuerda siempre consumir estos alimentos en las porciones adecuadas y siguiendo la secuencia alimentaria: primero los vegetales, luego las proteínas y al final los carbohidratos. Esto puede ayudar a reducir el pico glucémico posprandial. 
-Fuente: Tabla Peruana de Composición de Alimentos (TPCA) 2025, CENAN/INS, MINSA Perú.</t>
-        </is>
-      </c>
-      <c r="G41" t="n">
-        <v>0.8355</v>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>La quinua contiene 317 kcal por 100g según la TPCA CENAN/INS. El tarwi contiene 366 kcal por 100g según la TPCA CENAN/INS. La kiwicha contiene 351 kcal por 100g según la TPCA CENAN/INS.
+Para pacientes con Diabetes Mellitus Tipo 2 (DM2), te recomiendo el tarwi. Tiene un Índice Glucémico (IG) de 15, lo que significa que su impacto en la glucosa en sangre es muy bajo. Además, es rico en proteínas y fibra, lo que ayuda a regular la absorción de azúcar en el organismo. 
+La quinua y la kiwicha también son buenas opciones, pero el tarwi destaca por su bajo IG y su alto contenido proteico. ¡Excelente decisión al considerar estos superalimentos andinos!</t>
+        </is>
       </c>
       <c r="H41" t="n">
-        <v>5</v>
+        <v>0.633</v>
       </c>
       <c r="I41" t="n">
-        <v>3452</v>
+        <v>10</v>
       </c>
       <c r="J41" t="n">
-        <v>448</v>
+        <v>4738</v>
       </c>
       <c r="K41" t="n">
-        <v>25271</v>
+        <v>179</v>
+      </c>
+      <c r="L41" t="n">
+        <v>9730</v>
       </c>
     </row>
     <row r="42">
@@ -2602,30 +2652,34 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
           <t>El brócoli crudo contiene 34 kcal por 100g según la TPCA. IG 10, muy bajo. Aporta 3.6g de proteínas, 2.6g de fibra y vitamina C. RECOMENDADO de consumo libre para DM2. Sin restricción de cantidad.</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>El brócoli crudo tiene 32.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.
-Además, es considerado un alimento RECOMENDADO para pacientes con diabetes mellitus tipo 2. Esto se debe a que tiene un bajo contenido de carbohidratos (4.0g totales, 3.3g disponibles por cada 100g), y aporta una buena cantidad de fibra dietaria (0.7g por cada 100g), lo que ayuda a ralentizar la absorción de glucosa y a controlar los niveles de azúcar en sangre.
-Por lo tanto, el brócoli puede ser consumido de manera regular en la dieta de una persona con diabetes tipo 2. Sin embargo, como con cualquier alimento, es importante mantener una dieta equilibrada y variada. Te recomendaría que lo combines con otras verduras y alimentos ricos en proteínas y fibra para una alimentación saludable.</t>
-        </is>
-      </c>
-      <c r="G42" t="n">
-        <v>0.8155</v>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>El brócoli contiene 32.0 kcal por 100g según la TPCA CENAN/INS. 
+Además, el brócoli es un alimento recomendado para personas con diabetes mellitus tipo 2, ya que tiene un bajo contenido de carbohidratos y un índice glucémico bajo. Esto significa que puedes incluirlo en tu dieta de manera regular. ¡Es una excelente opción para tus comidas! 🥦</t>
+        </is>
       </c>
       <c r="H42" t="n">
-        <v>5</v>
+        <v>0.4795</v>
       </c>
       <c r="I42" t="n">
-        <v>3503</v>
+        <v>9</v>
       </c>
       <c r="J42" t="n">
-        <v>244</v>
+        <v>4063</v>
       </c>
       <c r="K42" t="n">
-        <v>9147</v>
+        <v>87</v>
+      </c>
+      <c r="L42" t="n">
+        <v>7597.9</v>
       </c>
     </row>
     <row r="43">
@@ -2643,35 +2697,38 @@
         <v>26</v>
       </c>
       <c r="D43" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
           <t>La espinaca cruda contiene 26 kcal por 100g según la TPCA. IG 15, muy bajo. Aporta 2.9g de proteínas, 2.2g de fibra y hierro. RECOMENDADO de consumo libre para DM2. Consumo ilimitado recomendado.</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>La espinaca cruda es un alimento muy nutritivo y bajo en calorías. Según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS, 100g de espinaca cruda aporta aproximadamente 30.0 kcal. 
-En cuanto a la cantidad de espinaca que puede comer un paciente con diabetes tipo 2, no hay un límite específico. La espinaca es rica en fibra dietaria (2.8g por 100g) y tiene un Índice Glucémico (IG) muy bajo de 15, lo que significa que su consumo no provoca picos bruscos en los niveles de azúcar en sangre. 
-Además, la espinaca es una excelente fuente de vitaminas y minerales, como el hierro (21.29mg por 100g), que es esencial para la producción de glóbulos rojos y el transporte de oxígeno en el cuerpo.
-Por lo tanto, la espinaca cruda puede ser incluida en la dieta de un paciente con diabetes tipo 2 de manera regular, siempre y cuando se mantenga una alimentación equilibrada y variada. Recuerda que cada paciente es único y puede tener necesidades nutricionales diferentes, por lo que siempre es recomendable consultar a un profesional de la salud antes de hacer cambios significativos en la dieta.</t>
-        </is>
-      </c>
-      <c r="G43" t="n">
-        <v>0.8205</v>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>La espinaca, hojas sin tallo, contiene 30.0 kcal por 100g según la TPCA CENAN/INS. 
+En cuanto a la cantidad que puede comer un diabético, la espinaca es una verdura muy baja en calorías y carbohidratos, por lo que se puede consumir en cantidades generosas. Sin embargo, es importante equilibrar la ingesta de otros alimentos en la comida. Generalmente, se recomienda que los vegetales ocupen la mayor parte del plato, así que puedes incluir una buena porción de espinaca en tus ensaladas o guisos. ¡Recuerda siempre seguir el orden de consumo recomendado!</t>
+        </is>
       </c>
       <c r="H43" t="n">
-        <v>5</v>
+        <v>0.509</v>
       </c>
       <c r="I43" t="n">
-        <v>3526</v>
+        <v>9</v>
       </c>
       <c r="J43" t="n">
-        <v>310</v>
+        <v>4201</v>
       </c>
       <c r="K43" t="n">
-        <v>21598</v>
+        <v>138</v>
+      </c>
+      <c r="L43" t="n">
+        <v>8432.4</v>
       </c>
     </row>
     <row r="44">
@@ -2693,31 +2750,34 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
           <t>La zanahoria cruda contiene 44 kcal por 100g según la TPCA. IG cruda 16, muy bajo. Aporta 1.1g de proteínas, 3.2g de fibra y betacarotenos. RECOMENDADO para DM2 cruda. Nota: cocida el IG sube a 47.</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>La zanahoria cruda tiene aproximadamente 19.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.
-Además, la zanahoria tiene un Índice Glucémico (IG) de 47, lo que se considera bajo. Esto significa que su consumo no provoca un aumento brusco de los niveles de glucosa en la sangre.
-Por lo tanto, las zanahorias crudas son aptas para pacientes con diabetes mellitus tipo 2 y pueden ser consumidas de forma moderada. Sin embargo, aunque su IG es bajo, no se deben consumir en exceso debido a su contenido de carbohidratos (7.6g por cada 100g). 
-Recuerda que es importante mantener una dieta equilibrada y variada, y siempre es recomendable consultar con tu médico o nutricionista antes de hacer cambios significativos en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G44" t="n">
-        <v>0.8287</v>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>La zanahoria contiene 19.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, la zanahoria es un alimento recomendado para personas con diabetes mellitus tipo 2, ya que tiene un Índice Glucémico (IG) de 47, lo que se considera bajo. Esto significa que su consumo no provoca picos significativos en los niveles de glucosa en sangre. Sin embargo, es importante consumirla en porciones adecuadas y dentro de un plan alimentario equilibrado. ¡Recuerda siempre consultar con tu médico o nutricionista sobre tu dieta!</t>
+        </is>
       </c>
       <c r="H44" t="n">
-        <v>5</v>
+        <v>0.4833</v>
       </c>
       <c r="I44" t="n">
-        <v>3531</v>
+        <v>7</v>
       </c>
       <c r="J44" t="n">
-        <v>231</v>
+        <v>3682</v>
       </c>
       <c r="K44" t="n">
-        <v>20571</v>
+        <v>124</v>
+      </c>
+      <c r="L44" t="n">
+        <v>6924.1</v>
       </c>
     </row>
     <row r="45">
@@ -2739,30 +2799,34 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
           <t>El jurel fresco contiene 124 kcal por 100g según la TPCA. IG 0. Aporta 20.2g de proteínas y 4.7g de grasas omega-3. RECOMENDADO para DM2. El omega-3 reduce inflamación y mejora la sensibilidad a la insulina.</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>El jurel fresco tiene 121.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Además, es muy recomendado para personas con diabetes tipo 2. Esto se debe a que tiene un Índice Glucémico (IG) de 0, lo que significa que no eleva rápidamente los niveles de azúcar en la sangre. También es una excelente fuente de proteínas (22.2g por cada 100g) y tiene un bajo contenido de grasa (2.7g por cada 100g). 
-Recuerda que una alimentación balanceada y el control de las porciones son clave para el manejo de la diabetes. Te sugiero que consultes con tu médico o nutricionista para un plan de alimentación personalizado.</t>
-        </is>
-      </c>
-      <c r="G45" t="n">
-        <v>0.8218</v>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>El jurel fresco contiene 121.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, el jurel fresco es bueno para diabéticos. Tiene un Índice Glucémico (IG) de 0, lo que significa que no eleva los niveles de glucosa en sangre. Además, es una excelente fuente de proteínas (22.2g por 100g) y contiene grasas saludables, lo que lo convierte en una opción nutritiva y recomendable para personas con Diabetes Mellitus Tipo 2.</t>
+        </is>
       </c>
       <c r="H45" t="n">
-        <v>5</v>
+        <v>0.5036</v>
       </c>
       <c r="I45" t="n">
-        <v>3447</v>
+        <v>8</v>
       </c>
       <c r="J45" t="n">
-        <v>199</v>
+        <v>3683</v>
       </c>
       <c r="K45" t="n">
-        <v>17096</v>
+        <v>111</v>
+      </c>
+      <c r="L45" t="n">
+        <v>7462.9</v>
       </c>
     </row>
     <row r="46">
@@ -2780,35 +2844,38 @@
         <v>121</v>
       </c>
       <c r="D46" t="n">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>La pechuga de pollo sin piel contiene 121 kcal por 100g según la TPCA. IG 0. Aporta 22.5g de proteínas y solo 2.8g de grasas. RECOMENDADO para DM2 como proteína magra. No eleva la glucosa.</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>La pechuga de pollo sin piel tiene aproximadamente 108.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS del Ministerio de Salud del Perú.
-Además, la pechuga de pollo sin piel es una excelente opción para las personas con diabetes tipo 2. Tiene un Índice Glucémico (IG) de 0, lo que significa que no eleva rápidamente los niveles de azúcar en la sangre. También es una buena fuente de proteínas (19.2g por cada 100g), lo que ayuda a mantener la sensación de saciedad y a controlar el peso.
-Recuerda siempre consumir la proteína (en este caso, la pechuga de pollo) después de los vegetales y antes de los carbohidratos, como parte de la secuenciación alimentaria recomendada para controlar mejor los niveles de glucosa en la sangre.
-¡Así que sí, la pechuga de pollo sin piel es apta y recomendada para la dieta de una persona con diabetes tipo 2!</t>
-        </is>
-      </c>
-      <c r="G46" t="n">
-        <v>0.8406</v>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>La pechuga de pollo sin piel contiene 121.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, es apta para la dieta del diabético. La pechuga de pollo es una fuente de proteína magra, baja en grasas y no contiene carbohidratos, lo que la convierte en una excelente opción para mantener estables los niveles de glucosa en sangre. Además, su alto contenido proteico ayuda a la saciedad. ¡Es una gran elección para tus comidas! 🍗</t>
+        </is>
       </c>
       <c r="H46" t="n">
-        <v>5</v>
+        <v>0.5896</v>
       </c>
       <c r="I46" t="n">
-        <v>3506</v>
+        <v>7</v>
       </c>
       <c r="J46" t="n">
-        <v>264</v>
+        <v>3518</v>
       </c>
       <c r="K46" t="n">
-        <v>20560</v>
+        <v>109</v>
+      </c>
+      <c r="L46" t="n">
+        <v>7479.5</v>
       </c>
     </row>
     <row r="47">
@@ -2830,31 +2897,34 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
           <t>El huevo de gallina crudo contiene 155 kcal por 100g (aprox. 1 huevo grande = 60g = 93 kcal) según la TPCA. Aporta 12.6g de proteínas, 11.5g de grasas y 0.7g de carbohidratos. IG 0. RECOMENDADO hasta 1 huevo diario para DM2. Proteína de alto valor biológico.</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>El huevo de gallina entero crudo tiene 166.0 kcal por cada 100g, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS. 
-En cuanto a la cantidad de huevos que puede comer un diabético por día, no existe un número exacto ya que depende de varios factores como el plan de alimentación individual, el nivel de actividad física y los niveles de glucosa en sangre. Sin embargo, el huevo es una excelente fuente de proteínas y tiene un Índice Glucémico (IG) de 0, lo que significa que no eleva rápidamente los niveles de glucosa en sangre. 
-Es importante recordar que aunque el huevo es saludable, la yema contiene grasas y colesterol, por lo que su consumo debe ser moderado. Una recomendación general podría ser consumir de 3 a 4 huevos enteros por semana, y si se desea consumir más, optar por las claras de huevo que son prácticamente pura proteína.
-Recuerda que cada persona es diferente y lo mejor es consultar con un profesional de la salud o un dietista registrado para obtener un plan de alimentación personalizado.</t>
-        </is>
-      </c>
-      <c r="G47" t="n">
-        <v>0.8315</v>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>El huevo de gallina entero, crudo, contiene 166.0 kcal por 100g según la TPCA CENAN/INS.
+En cuanto a la cantidad que puede consumir un diabético, generalmente se recomienda incluir 1 a 2 huevos al día en una dieta equilibrada, dependiendo de su perfil nutricional y recomendaciones médicas. Es importante que consultes con tu médico o nutricionista para determinar la cantidad adecuada para ti, ya que esto puede variar según tus necesidades individuales y otros factores de salud. ¡Recuerda siempre priorizar una alimentación balanceada! 🍳</t>
+        </is>
       </c>
       <c r="H47" t="n">
-        <v>5</v>
+        <v>0.5498</v>
       </c>
       <c r="I47" t="n">
-        <v>3496</v>
+        <v>6</v>
       </c>
       <c r="J47" t="n">
-        <v>274</v>
+        <v>3283</v>
       </c>
       <c r="K47" t="n">
-        <v>18736</v>
+        <v>118</v>
+      </c>
+      <c r="L47" t="n">
+        <v>7741.6</v>
       </c>
     </row>
     <row r="48">
@@ -2872,33 +2942,38 @@
         <v>347</v>
       </c>
       <c r="D48" t="n">
-        <v>343</v>
+        <v>347</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
           <t>El frijol canario crudo contiene 347 kcal por 100g según la TPCA. IG 31, bajo. Aporta 22.6g de proteínas, 1.5g de grasas y 66.4g de carbohidratos. Tiene 15.2g de fibra. RECOMENDADO para DM2. Consumir cocido 3 veces/semana.</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>[Similitud: 0.90] Alimento peruano: Frijol canario, crudo. Categoría TPCA: Leguminosas y derivados. Código: B 12. Composición por 100g de porción comestible: Energía 343.0 kcal. Proteínas 22.0g. Grasas 1.0g. Carbohidratos totales 62.0g. Fibra dietaria 15.0g. Agua 11.0g. Calcio 140.0mg. Hierro 6.0mg. Vitamina C 0.0mg. Fósforo 410.0mg. Índice Glucémico (IG): 31. IG bajo, recomendado para diabetes. Clasificación DM2: RECOMENDADO. Apto para pacientes con diabetes mellitus tipo 2. Fuente: Tabla Peruana de Composición de Alimentos (TPCA) 2025, CENAN/INS, MINSA Perú.
-El frijol canario es una excelente opción para personas con diabetes tipo 2. Tiene un Índice Glucémico (IG) bajo de 31, lo que significa que su consumo no provoca picos bruscos de glucosa en la sangre. Además, es rico en proteínas (22g por cada 100g) y fibra dietaria (15g por cada 100g), nutrientes que ayudan a controlar los niveles de azúcar en la sangre y a mantener la sensación de saciedad. Sin embargo, recuerda que contiene 62g de carbohidratos por cada 100g, por lo que debes controlar la porción para no exceder la cantidad de carbohidratos recomendada por comida (45g para este paciente).</t>
-        </is>
-      </c>
-      <c r="G48" t="n">
-        <v>0.823</v>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>El frijol canario crudo contiene 347.0 kcal por 100g según la TPCA CENAN/INS. 
+Es una excelente opción para personas con diabetes, ya que tiene un Índice Glucémico (IG) de 31, lo que lo clasifica como muy bajo. Esto significa que su consumo no provoca un aumento significativo en los niveles de glucosa en sangre. Además, es rico en proteínas (22.6g) y fibra (15.2g), lo que ayuda a mejorar la saciedad y a regular los niveles de azúcar en la sangre. ¡Una gran elección para tu alimentación!</t>
+        </is>
       </c>
       <c r="H48" t="n">
-        <v>5</v>
+        <v>0.5244</v>
       </c>
       <c r="I48" t="n">
-        <v>3431</v>
+        <v>9</v>
       </c>
       <c r="J48" t="n">
-        <v>404</v>
+        <v>4320</v>
       </c>
       <c r="K48" t="n">
-        <v>23486</v>
+        <v>130</v>
+      </c>
+      <c r="L48" t="n">
+        <v>7288.1</v>
       </c>
     </row>
     <row r="49">
@@ -2920,31 +2995,34 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
           <t>El maíz fresco o choclo contiene 104 kcal por 100g según la TPCA. IG 52, moderado. Aporta 3.3g de proteínas, 0.8g de grasas y 27.8g de carbohidratos. RECOMENDADO en porciones controladas para DM2. Máximo 1 choclo mediano (150g) por comida.</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>El maíz fresco, también conocido como choclo en Perú, tiene aproximadamente 104.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Además, el choclo tiene un Índice Glucémico (IG) de 52, que es considerado bajo (≤55). Esto significa que su consumo no eleva rápidamente los niveles de glucosa en la sangre, lo cual es beneficioso para las personas con diabetes tipo 2.
-Por lo tanto, sí, una persona con diabetes tipo 2 puede incluir choclo en su dieta, siempre y cuando se tenga en cuenta la cantidad consumida y se combine con otros alimentos saludables. Recuerda que el control de las porciones es clave, y en este caso, el choclo aporta alrededor de 25.1g de carbohidratos disponibles por cada 100g.
-Es importante que consultes con tu médico o un dietista registrado para obtener recomendaciones de alimentación personalizadas.</t>
-        </is>
-      </c>
-      <c r="G49" t="n">
-        <v>0.8433</v>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>El choclo o maíz fresco contiene 104.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, el maíz fresco es apto para pacientes con diabetes mellitus tipo 2, ya que tiene un Índice Glucémico (IG) de 52, lo que se considera bajo. Esto significa que su consumo no provocará un aumento significativo en los niveles de glucosa en sangre. Sin embargo, es importante controlar las porciones y combinarlo adecuadamente con otros alimentos.</t>
+        </is>
       </c>
       <c r="H49" t="n">
-        <v>5</v>
+        <v>0.5591</v>
       </c>
       <c r="I49" t="n">
-        <v>3493</v>
+        <v>9</v>
       </c>
       <c r="J49" t="n">
-        <v>249</v>
+        <v>4344</v>
       </c>
       <c r="K49" t="n">
-        <v>16261</v>
+        <v>107</v>
+      </c>
+      <c r="L49" t="n">
+        <v>6802</v>
       </c>
     </row>
     <row r="50">
@@ -2966,31 +3044,34 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
           <t>El arroz pilado cocido contiene 115 kcal por 100g según la TPCA. IG 73, alto. Aporta 2.4g de proteínas, 0.1g de grasas y 25.2g de carbohidratos. LIMITAR para DM2 por su IG alto. Preferir quinua (IG 53) o cebada (IG 28) como alternativa.</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>El arroz pilado cocido tiene 115.0 kcal por cada 100g de porción comestible, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-En cuanto a su consumo en pacientes con diabetes tipo 2, es importante tener en cuenta que el arroz pilado cocido tiene un Índice Glucémico (IG) de 73, lo cual es considerado alto. Esto significa que puede elevar rápidamente los niveles de glucosa en la sangre. Por lo tanto, su consumo debe ser limitado y siempre en combinación con alimentos de IG bajo y alto contenido de fibra para balancear el efecto en la glucosa.
-Recuerda que la cantidad de arroz en una comida debe ser moderada, no más de una pequeña taza, y siempre es mejor si se consume al final de la comida, después de las verduras y proteínas, siguiendo la secuenciación alimentaria. Esto puede ayudar a reducir el pico glucémico posprandial. 
-Siempre es importante que consultes a tu médico o nutricionista antes de hacer cambios en tu dieta.</t>
-        </is>
-      </c>
-      <c r="G50" t="n">
-        <v>0.8267</v>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>El arroz pilado cocido contiene 115.0 kcal por 100g según la TPCA CENAN/INS. 
+Sin embargo, es importante tener en cuenta que el arroz pilado tiene un Índice Glucémico (IG) de 73, lo que lo clasifica como un alimento de IG alto. Por lo tanto, se recomienda limitar su consumo en pacientes con diabetes tipo 2. Si decides incluirlo en tu dieta, es fundamental hacerlo con moderación y en porciones controladas, siempre acompañado de vegetales y proteínas para ayudar a reducir el pico glucémico. ¡Consulta con tu médico antes de hacer cambios en tu alimentación!</t>
+        </is>
       </c>
       <c r="H50" t="n">
-        <v>5</v>
+        <v>0.5115</v>
       </c>
       <c r="I50" t="n">
-        <v>3487</v>
+        <v>9</v>
       </c>
       <c r="J50" t="n">
-        <v>259</v>
+        <v>4338</v>
       </c>
       <c r="K50" t="n">
-        <v>22645</v>
+        <v>135</v>
+      </c>
+      <c r="L50" t="n">
+        <v>7761.3</v>
       </c>
     </row>
     <row r="51">
@@ -3008,34 +3089,38 @@
         <v>62</v>
       </c>
       <c r="D51" t="n">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
+          <t>contexto</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
           <t>La leche fresca de vaca entera contiene 62 kcal por 100g según la TPCA. IG 27, bajo. Aporta 3.2g de proteínas, 3.5g de grasas y 4.7g de carbohidratos (lactosa). RECOMENDADO para DM2 en porción de 1 vaso (200ml = ~125 kcal) por día.</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>La leche fresca de vaca entera tiene aproximadamente 63.0 kcal por cada 100g, según la Tabla Peruana de Composición de Alimentos (TPCA) del CENAN/INS.
-Sí, un paciente con diabetes tipo 2 puede consumirla. La leche fresca de vaca entera tiene un Índice Glucémico (IG) de 27, lo cual es considerado bajo. Los alimentos con IG bajo (≤55) son recomendados para personas con diabetes tipo 2 ya que provocan un aumento más lento y gradual de la glucosa en sangre.
-Recuerda siempre consumir en porciones moderadas y en el marco de una dieta equilibrada. Si tienes alguna duda, te recomiendo que consultes con tu médico o nutricionista.</t>
-        </is>
-      </c>
-      <c r="G51" t="n">
-        <v>0.8431</v>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>La leche fresca de vaca entera contiene 63.0 kcal por 100g según la TPCA CENAN/INS. 
+Sí, un diabético puede beber leche fresca de vaca entera, ya que tiene un Índice Glucémico (IG) de 27, lo cual es considerado bajo y recomendado para personas con diabetes mellitus tipo 2. Además, aporta proteínas y calcio, lo que puede ser beneficioso en una dieta equilibrada. Sin embargo, es importante consumirla con moderación y dentro del contexto de una alimentación balanceada. Siempre consulta con tu médico antes de hacer cambios en tu dieta.</t>
+        </is>
       </c>
       <c r="H51" t="n">
-        <v>5</v>
+        <v>0.5003</v>
       </c>
       <c r="I51" t="n">
-        <v>3473</v>
+        <v>9</v>
       </c>
       <c r="J51" t="n">
-        <v>183</v>
+        <v>4261</v>
       </c>
       <c r="K51" t="n">
-        <v>14058</v>
+        <v>129</v>
+      </c>
+      <c r="L51" t="n">
+        <v>7271.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>